<commit_message>
Rename pack to DogePack Classic Beta
Updated the resource pack metadata to point at the DogePack Classic 11 Beta directory and moved the bundled asset tree under that new name. This also replaces the old custom logo with the DogePack variant and refreshes the version guide spreadsheet.
</commit_message>
<xml_diff>
--- a/version_guide.xlsx
+++ b/version_guide.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\PrismLauncher\instances\NeoBeta Remastered\minecraft\resourcepacks\Classic-Reimagined\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{90EF5E16-4215-4E1A-865F-9BAB354A562A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{847E9376-A881-41CF-B8F4-9A3234E70852}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="521" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="230" uniqueCount="73">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="228" uniqueCount="73">
   <si>
     <t>Current version in development</t>
   </si>
@@ -492,6 +492,15 @@
     <xf numFmtId="1" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -544,15 +553,6 @@
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -745,7 +745,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:K79"/>
+  <dimension ref="A1:K77"/>
   <sheetFormatPr defaultColWidth="27.28515625" defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="36.5703125" style="6" customWidth="1"/>
@@ -754,20 +754,20 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A1" s="24" t="s">
+      <c r="A1" s="27" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="25"/>
-      <c r="C1" s="25"/>
-      <c r="D1" s="25"/>
-      <c r="E1" s="26"/>
-      <c r="G1" s="42" t="s">
+      <c r="B1" s="28"/>
+      <c r="C1" s="28"/>
+      <c r="D1" s="28"/>
+      <c r="E1" s="29"/>
+      <c r="G1" s="25" t="s">
         <v>66</v>
       </c>
-      <c r="H1" s="42"/>
-      <c r="I1" s="42"/>
-      <c r="J1" s="42"/>
-      <c r="K1" s="42"/>
+      <c r="H1" s="25"/>
+      <c r="I1" s="25"/>
+      <c r="J1" s="25"/>
+      <c r="K1" s="25"/>
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A2" s="21" t="s">
@@ -865,11 +865,11 @@
       <c r="K6" s="14"/>
     </row>
     <row r="7" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A7" s="33" t="s">
+      <c r="A7" s="36" t="s">
         <v>2</v>
       </c>
-      <c r="B7" s="34"/>
-      <c r="C7" s="35"/>
+      <c r="B7" s="37"/>
+      <c r="C7" s="38"/>
       <c r="D7" s="8" t="s">
         <v>3</v>
       </c>
@@ -887,27 +887,35 @@
       <c r="J7" s="13"/>
     </row>
     <row r="8" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A8" s="36" t="str">
+      <c r="A8" s="39" t="str">
         <f>G4 &amp; "." &amp; H4 &amp; "_" &amp; I4 &amp; "-build-" &amp; D8</f>
         <v>v10.0.11_3-build-6309-rt6</v>
       </c>
-      <c r="B8" s="37"/>
-      <c r="C8" s="38"/>
+      <c r="B8" s="40"/>
+      <c r="C8" s="41"/>
       <c r="D8" s="9" t="str">
         <f>B6&amp;"-rt"&amp;B2</f>
         <v>6309-rt6</v>
       </c>
       <c r="E8" s="18">
-        <f>K11</f>
-        <v>26.2</v>
-      </c>
-      <c r="G8" s="42" t="s">
-        <v>66</v>
-      </c>
-      <c r="H8" s="42"/>
-      <c r="I8" s="42"/>
-      <c r="J8" s="42"/>
-      <c r="K8" s="42"/>
+        <f>K9</f>
+        <v>26.3</v>
+      </c>
+      <c r="G8" s="8" t="s">
+        <v>2</v>
+      </c>
+      <c r="H8" s="8" t="s">
+        <v>6</v>
+      </c>
+      <c r="I8" s="8" t="s">
+        <v>7</v>
+      </c>
+      <c r="J8" s="8" t="s">
+        <v>3</v>
+      </c>
+      <c r="K8" s="8" t="s">
+        <v>4</v>
+      </c>
     </row>
     <row r="9" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A9" s="19" t="s">
@@ -916,852 +924,829 @@
       <c r="B9" s="20" t="s">
         <v>9</v>
       </c>
-      <c r="C9" s="27" t="s">
+      <c r="C9" s="30" t="s">
         <v>10</v>
       </c>
-      <c r="D9" s="28"/>
-      <c r="E9" s="29"/>
-      <c r="G9" s="7" t="s">
-        <v>5</v>
+      <c r="D9" s="31"/>
+      <c r="E9" s="32"/>
+      <c r="G9" s="9" t="s">
+        <v>11</v>
+      </c>
+      <c r="H9" s="9">
+        <v>11</v>
+      </c>
+      <c r="I9" s="9">
+        <v>2</v>
+      </c>
+      <c r="J9" s="9" t="str">
+        <f>J4</f>
+        <v>6309-rt6</v>
+      </c>
+      <c r="K9" s="9">
+        <v>26.3</v>
       </c>
     </row>
     <row r="10" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A10" s="6" t="s">
         <v>68</v>
       </c>
-      <c r="C10" s="30" t="s">
+      <c r="C10" s="33" t="s">
         <v>12</v>
       </c>
-      <c r="D10" s="31"/>
-      <c r="E10" s="32"/>
-      <c r="G10" s="8" t="s">
-        <v>2</v>
-      </c>
-      <c r="H10" s="8" t="s">
-        <v>6</v>
-      </c>
-      <c r="I10" s="8" t="s">
-        <v>7</v>
-      </c>
-      <c r="J10" s="8" t="s">
-        <v>3</v>
-      </c>
-      <c r="K10" s="8" t="s">
-        <v>4</v>
-      </c>
+      <c r="D10" s="34"/>
+      <c r="E10" s="35"/>
+      <c r="G10" s="10" t="s">
+        <v>13</v>
+      </c>
+      <c r="H10" s="11" t="str">
+        <f>H5</f>
+        <v>DogePack_Classic_11_Beta</v>
+      </c>
+      <c r="I10" s="12"/>
+      <c r="J10" s="13"/>
+      <c r="K10" s="14"/>
     </row>
     <row r="11" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A11" s="6" t="s">
         <v>69</v>
       </c>
-      <c r="G11" s="9" t="s">
-        <v>11</v>
-      </c>
-      <c r="H11" s="9">
-        <v>11</v>
-      </c>
-      <c r="I11" s="9">
-        <v>2</v>
-      </c>
-      <c r="J11" s="9" t="str">
-        <f>J4</f>
-        <v>6309-rt6</v>
-      </c>
-      <c r="K11" s="9">
-        <v>26.2</v>
-      </c>
+      <c r="G11" s="10" t="s">
+        <v>14</v>
+      </c>
+      <c r="H11" s="11" t="str">
+        <f>G9 &amp; "." &amp; H9 &amp; "_" &amp; I9 &amp; "-" &amp; H10</f>
+        <v>v10.0.11_2-DogePack_Classic_11_Beta</v>
+      </c>
+      <c r="I11" s="12"/>
+      <c r="J11" s="13"/>
+      <c r="K11" s="14"/>
     </row>
     <row r="12" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A12" s="6" t="s">
         <v>70</v>
       </c>
       <c r="G12" s="10" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="H12" s="11" t="str">
-        <f>"Classic_Reimagined_11" &amp; G9</f>
-        <v>Classic_Reimagined_11_SE_2.1</v>
+        <f>H11 &amp; "-build-" &amp; J9</f>
+        <v>v10.0.11_2-DogePack_Classic_11_Beta-build-6309-rt6</v>
       </c>
       <c r="I12" s="12"/>
       <c r="J12" s="13"/>
-      <c r="K12" s="14"/>
     </row>
     <row r="13" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A13" s="6" t="s">
         <v>72</v>
       </c>
-      <c r="G13" s="10" t="s">
+      <c r="G13" s="26" t="s">
+        <v>1</v>
+      </c>
+      <c r="H13" s="26"/>
+      <c r="I13" s="26"/>
+      <c r="J13" s="26"/>
+      <c r="K13" s="26"/>
+    </row>
+    <row r="14" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="G14" s="7" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="15" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="G15" s="8" t="s">
+        <v>2</v>
+      </c>
+      <c r="H15" s="8" t="s">
+        <v>6</v>
+      </c>
+      <c r="I15" s="8" t="s">
+        <v>7</v>
+      </c>
+      <c r="J15" s="8" t="s">
+        <v>3</v>
+      </c>
+      <c r="K15" s="8" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="16" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="G16" s="9" t="s">
+        <v>11</v>
+      </c>
+      <c r="H16" s="9">
+        <v>11</v>
+      </c>
+      <c r="I16" s="9">
+        <v>1</v>
+      </c>
+      <c r="J16" s="9" t="str">
+        <f>J9</f>
+        <v>6309-rt6</v>
+      </c>
+      <c r="K16" s="9">
+        <v>26.1</v>
+      </c>
+    </row>
+    <row r="17" spans="7:11" x14ac:dyDescent="0.3">
+      <c r="G17" s="10" t="s">
+        <v>13</v>
+      </c>
+      <c r="H17" s="11" t="str">
+        <f>"Classic_Reimagined_10" &amp; G14</f>
+        <v>Classic_Reimagined_10_SE_2.1</v>
+      </c>
+      <c r="I17" s="12"/>
+      <c r="J17" s="13"/>
+      <c r="K17" s="14"/>
+    </row>
+    <row r="18" spans="7:11" x14ac:dyDescent="0.3">
+      <c r="G18" s="10" t="s">
         <v>14</v>
       </c>
-      <c r="H13" s="11" t="str">
-        <f>G11 &amp; "." &amp; H11 &amp; "_" &amp; I11 &amp; "-" &amp; H12</f>
-        <v>v10.0.11_2-Classic_Reimagined_11_SE_2.1</v>
-      </c>
-      <c r="I13" s="12"/>
-      <c r="J13" s="13"/>
-      <c r="K13" s="14"/>
-    </row>
-    <row r="14" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="G14" s="10" t="s">
-        <v>15</v>
-      </c>
-      <c r="H14" s="11" t="str">
-        <f>H13 &amp; "-build-" &amp; J11</f>
-        <v>v10.0.11_2-Classic_Reimagined_11_SE_2.1-build-6309-rt6</v>
-      </c>
-      <c r="I14" s="12"/>
-      <c r="J14" s="13"/>
-    </row>
-    <row r="15" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="G15" s="43" t="s">
-        <v>1</v>
-      </c>
-      <c r="H15" s="43"/>
-      <c r="I15" s="43"/>
-      <c r="J15" s="43"/>
-      <c r="K15" s="43"/>
-    </row>
-    <row r="16" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="G16" s="7" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="17" spans="7:11" x14ac:dyDescent="0.3">
-      <c r="G17" s="8" t="s">
-        <v>2</v>
-      </c>
-      <c r="H17" s="8" t="s">
-        <v>6</v>
-      </c>
-      <c r="I17" s="8" t="s">
-        <v>7</v>
-      </c>
-      <c r="J17" s="8" t="s">
-        <v>3</v>
-      </c>
-      <c r="K17" s="8" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="18" spans="7:11" x14ac:dyDescent="0.3">
-      <c r="G18" s="9" t="s">
-        <v>11</v>
-      </c>
-      <c r="H18" s="9">
-        <v>11</v>
-      </c>
-      <c r="I18" s="9">
-        <v>1</v>
-      </c>
-      <c r="J18" s="9" t="str">
-        <f>J11</f>
-        <v>6309-rt6</v>
-      </c>
-      <c r="K18" s="9">
-        <v>26.1</v>
-      </c>
+      <c r="H18" s="11" t="str">
+        <f>G16 &amp; "." &amp; H16 &amp; "_" &amp; I16 &amp; "-" &amp; H17</f>
+        <v>v10.0.11_1-Classic_Reimagined_10_SE_2.1</v>
+      </c>
+      <c r="I18" s="12"/>
+      <c r="J18" s="13"/>
+      <c r="K18" s="14"/>
     </row>
     <row r="19" spans="7:11" x14ac:dyDescent="0.3">
       <c r="G19" s="10" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="H19" s="11" t="str">
-        <f>"Classic_Reimagined_10" &amp; G16</f>
-        <v>Classic_Reimagined_10_SE_2.1</v>
+        <f>H18 &amp; "-build-" &amp; J16</f>
+        <v>v10.0.11_1-Classic_Reimagined_10_SE_2.1-build-6309-rt6</v>
       </c>
       <c r="I19" s="12"/>
       <c r="J19" s="13"/>
-      <c r="K19" s="14"/>
     </row>
     <row r="20" spans="7:11" x14ac:dyDescent="0.3">
-      <c r="G20" s="10" t="s">
+      <c r="G20" s="7" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="21" spans="7:11" x14ac:dyDescent="0.3">
+      <c r="G21" s="8" t="s">
+        <v>17</v>
+      </c>
+      <c r="H21" s="8" t="s">
+        <v>6</v>
+      </c>
+      <c r="I21" s="8" t="s">
+        <v>3</v>
+      </c>
+      <c r="J21" s="8" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="22" spans="7:11" x14ac:dyDescent="0.3">
+      <c r="G22" s="9" t="s">
+        <v>11</v>
+      </c>
+      <c r="H22" s="9">
+        <v>10</v>
+      </c>
+      <c r="I22" s="9" t="str">
+        <f>J16</f>
+        <v>6309-rt6</v>
+      </c>
+      <c r="J22" s="9" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="23" spans="7:11" x14ac:dyDescent="0.3">
+      <c r="G23" s="10" t="s">
+        <v>13</v>
+      </c>
+      <c r="H23" s="15" t="str">
+        <f>"Classic_Reimagined_10" &amp; G20</f>
+        <v>Classic_Reimagined_10_SE_2</v>
+      </c>
+      <c r="I23" s="16"/>
+      <c r="J23" s="14"/>
+    </row>
+    <row r="24" spans="7:11" x14ac:dyDescent="0.3">
+      <c r="G24" s="10" t="s">
         <v>14</v>
       </c>
-      <c r="H20" s="11" t="str">
-        <f>G18 &amp; "." &amp; H18 &amp; "_" &amp; I18 &amp; "-" &amp; H19</f>
-        <v>v10.0.11_1-Classic_Reimagined_10_SE_2.1</v>
-      </c>
-      <c r="I20" s="12"/>
-      <c r="J20" s="13"/>
-      <c r="K20" s="14"/>
-    </row>
-    <row r="21" spans="7:11" x14ac:dyDescent="0.3">
-      <c r="G21" s="10" t="s">
-        <v>15</v>
-      </c>
-      <c r="H21" s="11" t="str">
-        <f>H20 &amp; "-build-" &amp; J18</f>
-        <v>v10.0.11_1-Classic_Reimagined_10_SE_2.1-build-6309-rt6</v>
-      </c>
-      <c r="I21" s="12"/>
-      <c r="J21" s="13"/>
-    </row>
-    <row r="22" spans="7:11" x14ac:dyDescent="0.3">
-      <c r="G22" s="7" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="23" spans="7:11" x14ac:dyDescent="0.3">
-      <c r="G23" s="8" t="s">
-        <v>17</v>
-      </c>
-      <c r="H23" s="8" t="s">
-        <v>6</v>
-      </c>
-      <c r="I23" s="8" t="s">
-        <v>3</v>
-      </c>
-      <c r="J23" s="8" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="24" spans="7:11" x14ac:dyDescent="0.3">
-      <c r="G24" s="9" t="s">
-        <v>11</v>
-      </c>
-      <c r="H24" s="9">
-        <v>10</v>
-      </c>
-      <c r="I24" s="9" t="str">
-        <f>J18</f>
-        <v>6309-rt6</v>
-      </c>
-      <c r="J24" s="9" t="s">
-        <v>18</v>
-      </c>
+      <c r="H24" s="15" t="str">
+        <f>G22 &amp; "." &amp; H22 &amp; "-" &amp; H23</f>
+        <v>v10.0.10-Classic_Reimagined_10_SE_2</v>
+      </c>
+      <c r="I24" s="16"/>
+      <c r="J24" s="14"/>
     </row>
     <row r="25" spans="7:11" x14ac:dyDescent="0.3">
       <c r="G25" s="10" t="s">
+        <v>15</v>
+      </c>
+      <c r="H25" s="15" t="str">
+        <f>H24 &amp; "-build-" &amp; I22</f>
+        <v>v10.0.10-Classic_Reimagined_10_SE_2-build-6309-rt6</v>
+      </c>
+      <c r="I25" s="16"/>
+    </row>
+    <row r="26" spans="7:11" x14ac:dyDescent="0.3">
+      <c r="G26" s="8" t="s">
+        <v>17</v>
+      </c>
+      <c r="H26" s="8" t="s">
+        <v>6</v>
+      </c>
+      <c r="I26" s="8" t="s">
+        <v>3</v>
+      </c>
+      <c r="J26" s="8" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="27" spans="7:11" x14ac:dyDescent="0.3">
+      <c r="G27" s="9" t="s">
+        <v>11</v>
+      </c>
+      <c r="H27" s="9">
+        <v>9</v>
+      </c>
+      <c r="I27" s="9" t="str">
+        <f>I22</f>
+        <v>6309-rt6</v>
+      </c>
+      <c r="J27" s="9" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="28" spans="7:11" x14ac:dyDescent="0.3">
+      <c r="G28" s="10" t="s">
         <v>13</v>
       </c>
-      <c r="H25" s="15" t="str">
-        <f>"Classic_Reimagined_10" &amp; G22</f>
+      <c r="H28" s="15" t="str">
+        <f>H23</f>
         <v>Classic_Reimagined_10_SE_2</v>
       </c>
-      <c r="I25" s="16"/>
-      <c r="J25" s="14"/>
-    </row>
-    <row r="26" spans="7:11" x14ac:dyDescent="0.3">
-      <c r="G26" s="10" t="s">
+      <c r="I28" s="16"/>
+      <c r="J28" s="14"/>
+    </row>
+    <row r="29" spans="7:11" x14ac:dyDescent="0.3">
+      <c r="G29" s="10" t="s">
         <v>14</v>
       </c>
-      <c r="H26" s="15" t="str">
-        <f>G24 &amp; "." &amp; H24 &amp; "-" &amp; H25</f>
-        <v>v10.0.10-Classic_Reimagined_10_SE_2</v>
-      </c>
-      <c r="I26" s="16"/>
-      <c r="J26" s="14"/>
-    </row>
-    <row r="27" spans="7:11" x14ac:dyDescent="0.3">
-      <c r="G27" s="10" t="s">
-        <v>15</v>
-      </c>
-      <c r="H27" s="15" t="str">
-        <f>H26 &amp; "-build-" &amp; I24</f>
-        <v>v10.0.10-Classic_Reimagined_10_SE_2-build-6309-rt6</v>
-      </c>
-      <c r="I27" s="16"/>
-    </row>
-    <row r="28" spans="7:11" x14ac:dyDescent="0.3">
-      <c r="G28" s="8" t="s">
-        <v>17</v>
-      </c>
-      <c r="H28" s="8" t="s">
-        <v>6</v>
-      </c>
-      <c r="I28" s="8" t="s">
-        <v>3</v>
-      </c>
-      <c r="J28" s="8" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="29" spans="7:11" x14ac:dyDescent="0.3">
-      <c r="G29" s="9" t="s">
-        <v>11</v>
-      </c>
-      <c r="H29" s="9">
-        <v>9</v>
-      </c>
-      <c r="I29" s="9" t="str">
-        <f>I24</f>
-        <v>6309-rt6</v>
-      </c>
-      <c r="J29" s="9" t="s">
-        <v>19</v>
-      </c>
+      <c r="H29" s="15" t="str">
+        <f>G27 &amp; "." &amp; H27 &amp; "-" &amp; H28</f>
+        <v>v10.0.9-Classic_Reimagined_10_SE_2</v>
+      </c>
+      <c r="I29" s="16"/>
+      <c r="J29" s="14"/>
     </row>
     <row r="30" spans="7:11" x14ac:dyDescent="0.3">
       <c r="G30" s="10" t="s">
+        <v>15</v>
+      </c>
+      <c r="H30" s="15" t="str">
+        <f>H29 &amp; "-build-" &amp; I27</f>
+        <v>v10.0.9-Classic_Reimagined_10_SE_2-build-6309-rt6</v>
+      </c>
+      <c r="I30" s="16"/>
+    </row>
+    <row r="31" spans="7:11" x14ac:dyDescent="0.3">
+      <c r="G31" s="8" t="s">
+        <v>17</v>
+      </c>
+      <c r="H31" s="8" t="s">
+        <v>6</v>
+      </c>
+      <c r="I31" s="8" t="s">
+        <v>3</v>
+      </c>
+      <c r="J31" s="8" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="32" spans="7:11" x14ac:dyDescent="0.3">
+      <c r="G32" s="9" t="s">
+        <v>11</v>
+      </c>
+      <c r="H32" s="9">
+        <v>7</v>
+      </c>
+      <c r="I32" s="9" t="str">
+        <f>I27</f>
+        <v>6309-rt6</v>
+      </c>
+      <c r="J32" s="9" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="33" spans="7:10" x14ac:dyDescent="0.3">
+      <c r="G33" s="10" t="s">
         <v>13</v>
       </c>
-      <c r="H30" s="15" t="str">
-        <f>H25</f>
+      <c r="H33" s="15" t="str">
+        <f>H28</f>
         <v>Classic_Reimagined_10_SE_2</v>
       </c>
-      <c r="I30" s="16"/>
-      <c r="J30" s="14"/>
-    </row>
-    <row r="31" spans="7:11" x14ac:dyDescent="0.3">
-      <c r="G31" s="10" t="s">
+      <c r="I33" s="16"/>
+      <c r="J33" s="14"/>
+    </row>
+    <row r="34" spans="7:10" x14ac:dyDescent="0.3">
+      <c r="G34" s="10" t="s">
         <v>14</v>
       </c>
-      <c r="H31" s="15" t="str">
-        <f>G29 &amp; "." &amp; H29 &amp; "-" &amp; H30</f>
-        <v>v10.0.9-Classic_Reimagined_10_SE_2</v>
-      </c>
-      <c r="I31" s="16"/>
-      <c r="J31" s="14"/>
-    </row>
-    <row r="32" spans="7:11" x14ac:dyDescent="0.3">
-      <c r="G32" s="10" t="s">
-        <v>15</v>
-      </c>
-      <c r="H32" s="15" t="str">
-        <f>H31 &amp; "-build-" &amp; I29</f>
-        <v>v10.0.9-Classic_Reimagined_10_SE_2-build-6309-rt6</v>
-      </c>
-      <c r="I32" s="16"/>
-    </row>
-    <row r="33" spans="7:10" x14ac:dyDescent="0.3">
-      <c r="G33" s="8" t="s">
-        <v>17</v>
-      </c>
-      <c r="H33" s="8" t="s">
-        <v>6</v>
-      </c>
-      <c r="I33" s="8" t="s">
-        <v>3</v>
-      </c>
-      <c r="J33" s="8" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="34" spans="7:10" x14ac:dyDescent="0.3">
-      <c r="G34" s="9" t="s">
-        <v>11</v>
-      </c>
-      <c r="H34" s="9">
-        <v>7</v>
-      </c>
-      <c r="I34" s="9" t="str">
-        <f>I29</f>
-        <v>6309-rt6</v>
-      </c>
-      <c r="J34" s="9" t="s">
-        <v>20</v>
-      </c>
+      <c r="H34" s="15" t="str">
+        <f>G32 &amp; "." &amp; H32 &amp; "-" &amp; H33</f>
+        <v>v10.0.7-Classic_Reimagined_10_SE_2</v>
+      </c>
+      <c r="I34" s="16"/>
+      <c r="J34" s="14"/>
     </row>
     <row r="35" spans="7:10" x14ac:dyDescent="0.3">
       <c r="G35" s="10" t="s">
+        <v>15</v>
+      </c>
+      <c r="H35" s="15" t="str">
+        <f>H34 &amp; "-build-" &amp; I32</f>
+        <v>v10.0.7-Classic_Reimagined_10_SE_2-build-6309-rt6</v>
+      </c>
+      <c r="I35" s="16"/>
+    </row>
+    <row r="36" spans="7:10" x14ac:dyDescent="0.3">
+      <c r="G36" s="8" t="s">
+        <v>17</v>
+      </c>
+      <c r="H36" s="8" t="s">
+        <v>6</v>
+      </c>
+      <c r="I36" s="8" t="s">
+        <v>3</v>
+      </c>
+      <c r="J36" s="8" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="37" spans="7:10" x14ac:dyDescent="0.3">
+      <c r="G37" s="9" t="s">
+        <v>11</v>
+      </c>
+      <c r="H37" s="9">
+        <v>4</v>
+      </c>
+      <c r="I37" s="9" t="str">
+        <f>I32</f>
+        <v>6309-rt6</v>
+      </c>
+      <c r="J37" s="9" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="38" spans="7:10" x14ac:dyDescent="0.3">
+      <c r="G38" s="10" t="s">
         <v>13</v>
       </c>
-      <c r="H35" s="15" t="str">
-        <f>H30</f>
+      <c r="H38" s="15" t="str">
+        <f>H33</f>
         <v>Classic_Reimagined_10_SE_2</v>
       </c>
-      <c r="I35" s="16"/>
-      <c r="J35" s="14"/>
-    </row>
-    <row r="36" spans="7:10" x14ac:dyDescent="0.3">
-      <c r="G36" s="10" t="s">
+      <c r="I38" s="16"/>
+      <c r="J38" s="14"/>
+    </row>
+    <row r="39" spans="7:10" x14ac:dyDescent="0.3">
+      <c r="G39" s="10" t="s">
         <v>14</v>
       </c>
-      <c r="H36" s="15" t="str">
-        <f>G34 &amp; "." &amp; H34 &amp; "-" &amp; H35</f>
-        <v>v10.0.7-Classic_Reimagined_10_SE_2</v>
-      </c>
-      <c r="I36" s="16"/>
-      <c r="J36" s="14"/>
-    </row>
-    <row r="37" spans="7:10" x14ac:dyDescent="0.3">
-      <c r="G37" s="10" t="s">
-        <v>15</v>
-      </c>
-      <c r="H37" s="15" t="str">
-        <f>H36 &amp; "-build-" &amp; I34</f>
-        <v>v10.0.7-Classic_Reimagined_10_SE_2-build-6309-rt6</v>
-      </c>
-      <c r="I37" s="16"/>
-    </row>
-    <row r="38" spans="7:10" x14ac:dyDescent="0.3">
-      <c r="G38" s="8" t="s">
-        <v>17</v>
-      </c>
-      <c r="H38" s="8" t="s">
-        <v>6</v>
-      </c>
-      <c r="I38" s="8" t="s">
-        <v>3</v>
-      </c>
-      <c r="J38" s="8" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="39" spans="7:10" x14ac:dyDescent="0.3">
-      <c r="G39" s="9" t="s">
-        <v>11</v>
-      </c>
-      <c r="H39" s="9">
-        <v>4</v>
-      </c>
-      <c r="I39" s="9" t="str">
-        <f>I34</f>
-        <v>6309-rt6</v>
-      </c>
-      <c r="J39" s="9" t="s">
-        <v>21</v>
-      </c>
+      <c r="H39" s="15" t="str">
+        <f>G37 &amp; "." &amp; H37 &amp; "-" &amp; H38</f>
+        <v>v10.0.4-Classic_Reimagined_10_SE_2</v>
+      </c>
+      <c r="I39" s="16"/>
+      <c r="J39" s="14"/>
     </row>
     <row r="40" spans="7:10" x14ac:dyDescent="0.3">
       <c r="G40" s="10" t="s">
+        <v>15</v>
+      </c>
+      <c r="H40" s="15" t="str">
+        <f>H39 &amp; "-build-" &amp; I37</f>
+        <v>v10.0.4-Classic_Reimagined_10_SE_2-build-6309-rt6</v>
+      </c>
+      <c r="I40" s="16"/>
+    </row>
+    <row r="41" spans="7:10" x14ac:dyDescent="0.3">
+      <c r="G41" s="7" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="42" spans="7:10" x14ac:dyDescent="0.3">
+      <c r="G42" s="8" t="s">
+        <v>17</v>
+      </c>
+      <c r="H42" s="8" t="s">
+        <v>6</v>
+      </c>
+      <c r="I42" s="8" t="s">
+        <v>3</v>
+      </c>
+      <c r="J42" s="8" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="43" spans="7:10" x14ac:dyDescent="0.3">
+      <c r="G43" s="9" t="s">
+        <v>11</v>
+      </c>
+      <c r="H43" s="9">
+        <v>3</v>
+      </c>
+      <c r="I43" s="9" t="str">
+        <f>I37</f>
+        <v>6309-rt6</v>
+      </c>
+      <c r="J43" s="9" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="44" spans="7:10" x14ac:dyDescent="0.3">
+      <c r="G44" s="10" t="s">
         <v>13</v>
       </c>
-      <c r="H40" s="15" t="str">
-        <f>H35</f>
-        <v>Classic_Reimagined_10_SE_2</v>
-      </c>
-      <c r="I40" s="16"/>
-      <c r="J40" s="14"/>
-    </row>
-    <row r="41" spans="7:10" x14ac:dyDescent="0.3">
-      <c r="G41" s="10" t="s">
+      <c r="H44" s="15" t="str">
+        <f>"Classic_Reimagined_10" &amp; G41</f>
+        <v>Classic_Reimagined_10_SE</v>
+      </c>
+      <c r="I44" s="16"/>
+      <c r="J44" s="14"/>
+    </row>
+    <row r="45" spans="7:10" x14ac:dyDescent="0.3">
+      <c r="G45" s="10" t="s">
         <v>14</v>
       </c>
-      <c r="H41" s="15" t="str">
-        <f>G39 &amp; "." &amp; H39 &amp; "-" &amp; H40</f>
-        <v>v10.0.4-Classic_Reimagined_10_SE_2</v>
-      </c>
-      <c r="I41" s="16"/>
-      <c r="J41" s="14"/>
-    </row>
-    <row r="42" spans="7:10" x14ac:dyDescent="0.3">
-      <c r="G42" s="10" t="s">
-        <v>15</v>
-      </c>
-      <c r="H42" s="15" t="str">
-        <f>H41 &amp; "-build-" &amp; I39</f>
-        <v>v10.0.4-Classic_Reimagined_10_SE_2-build-6309-rt6</v>
-      </c>
-      <c r="I42" s="16"/>
-    </row>
-    <row r="43" spans="7:10" x14ac:dyDescent="0.3">
-      <c r="G43" s="7" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="44" spans="7:10" x14ac:dyDescent="0.3">
-      <c r="G44" s="8" t="s">
-        <v>17</v>
-      </c>
-      <c r="H44" s="8" t="s">
-        <v>6</v>
-      </c>
-      <c r="I44" s="8" t="s">
-        <v>3</v>
-      </c>
-      <c r="J44" s="8" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="45" spans="7:10" x14ac:dyDescent="0.3">
-      <c r="G45" s="9" t="s">
-        <v>11</v>
-      </c>
-      <c r="H45" s="9">
-        <v>3</v>
-      </c>
-      <c r="I45" s="9" t="str">
-        <f>I39</f>
-        <v>6309-rt6</v>
-      </c>
-      <c r="J45" s="9" t="s">
-        <v>23</v>
-      </c>
+      <c r="H45" s="15" t="str">
+        <f>G43 &amp; "." &amp; H43 &amp; "-" &amp; H44</f>
+        <v>v10.0.3-Classic_Reimagined_10_SE</v>
+      </c>
+      <c r="I45" s="16"/>
+      <c r="J45" s="14"/>
     </row>
     <row r="46" spans="7:10" x14ac:dyDescent="0.3">
       <c r="G46" s="10" t="s">
+        <v>15</v>
+      </c>
+      <c r="H46" s="15" t="str">
+        <f>H45 &amp; "-build-" &amp; I43</f>
+        <v>v10.0.3-Classic_Reimagined_10_SE-build-6309-rt6</v>
+      </c>
+      <c r="I46" s="16"/>
+    </row>
+    <row r="47" spans="7:10" x14ac:dyDescent="0.3">
+      <c r="G47" s="7" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="48" spans="7:10" x14ac:dyDescent="0.3">
+      <c r="G48" s="8" t="s">
+        <v>17</v>
+      </c>
+      <c r="H48" s="8" t="s">
+        <v>6</v>
+      </c>
+      <c r="I48" s="8" t="s">
+        <v>3</v>
+      </c>
+      <c r="J48" s="8" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="49" spans="7:10" x14ac:dyDescent="0.3">
+      <c r="G49" s="9" t="s">
+        <v>11</v>
+      </c>
+      <c r="H49" s="9">
+        <v>2</v>
+      </c>
+      <c r="I49" s="9" t="str">
+        <f>I43</f>
+        <v>6309-rt6</v>
+      </c>
+      <c r="J49" s="9" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="50" spans="7:10" x14ac:dyDescent="0.3">
+      <c r="G50" s="10" t="s">
         <v>13</v>
       </c>
-      <c r="H46" s="15" t="str">
-        <f>"Classic_Reimagined_10" &amp; G43</f>
-        <v>Classic_Reimagined_10_SE</v>
-      </c>
-      <c r="I46" s="16"/>
-      <c r="J46" s="14"/>
-    </row>
-    <row r="47" spans="7:10" x14ac:dyDescent="0.3">
-      <c r="G47" s="10" t="s">
+      <c r="H50" s="15" t="s">
+        <v>26</v>
+      </c>
+      <c r="I50" s="16"/>
+      <c r="J50" s="14"/>
+    </row>
+    <row r="51" spans="7:10" x14ac:dyDescent="0.3">
+      <c r="G51" s="10" t="s">
         <v>14</v>
       </c>
-      <c r="H47" s="15" t="str">
-        <f>G45 &amp; "." &amp; H45 &amp; "-" &amp; H46</f>
-        <v>v10.0.3-Classic_Reimagined_10_SE</v>
-      </c>
-      <c r="I47" s="16"/>
-      <c r="J47" s="14"/>
-    </row>
-    <row r="48" spans="7:10" x14ac:dyDescent="0.3">
-      <c r="G48" s="10" t="s">
-        <v>15</v>
-      </c>
-      <c r="H48" s="15" t="str">
-        <f>H47 &amp; "-build-" &amp; I45</f>
-        <v>v10.0.3-Classic_Reimagined_10_SE-build-6309-rt6</v>
-      </c>
-      <c r="I48" s="16"/>
-    </row>
-    <row r="49" spans="7:10" x14ac:dyDescent="0.3">
-      <c r="G49" s="7" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="50" spans="7:10" x14ac:dyDescent="0.3">
-      <c r="G50" s="8" t="s">
-        <v>17</v>
-      </c>
-      <c r="H50" s="8" t="s">
-        <v>6</v>
-      </c>
-      <c r="I50" s="8" t="s">
-        <v>3</v>
-      </c>
-      <c r="J50" s="8" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="51" spans="7:10" x14ac:dyDescent="0.3">
-      <c r="G51" s="9" t="s">
-        <v>11</v>
-      </c>
-      <c r="H51" s="9">
-        <v>2</v>
-      </c>
-      <c r="I51" s="9" t="str">
-        <f>I45</f>
-        <v>6309-rt6</v>
-      </c>
-      <c r="J51" s="9" t="s">
-        <v>25</v>
-      </c>
+      <c r="H51" s="15" t="str">
+        <f>G49 &amp; "." &amp; H49 &amp; "-" &amp; H50</f>
+        <v>v10.0.2-Classic_Reimagined_10s</v>
+      </c>
+      <c r="I51" s="16"/>
+      <c r="J51" s="14"/>
     </row>
     <row r="52" spans="7:10" x14ac:dyDescent="0.3">
       <c r="G52" s="10" t="s">
+        <v>15</v>
+      </c>
+      <c r="H52" s="15" t="str">
+        <f>H51 &amp; "-build-" &amp; I49</f>
+        <v>v10.0.2-Classic_Reimagined_10s-build-6309-rt6</v>
+      </c>
+      <c r="I52" s="16"/>
+    </row>
+    <row r="53" spans="7:10" x14ac:dyDescent="0.3">
+      <c r="G53" s="7" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="54" spans="7:10" x14ac:dyDescent="0.3">
+      <c r="G54" s="8" t="s">
+        <v>17</v>
+      </c>
+      <c r="H54" s="8" t="s">
+        <v>6</v>
+      </c>
+      <c r="I54" s="8" t="s">
+        <v>3</v>
+      </c>
+      <c r="J54" s="8" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="55" spans="7:10" x14ac:dyDescent="0.3">
+      <c r="G55" s="9" t="s">
+        <v>11</v>
+      </c>
+      <c r="H55" s="9">
+        <v>1</v>
+      </c>
+      <c r="I55" s="9" t="str">
+        <f>I49</f>
+        <v>6309-rt6</v>
+      </c>
+      <c r="J55" s="9" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="56" spans="7:10" x14ac:dyDescent="0.3">
+      <c r="G56" s="10" t="s">
         <v>13</v>
       </c>
-      <c r="H52" s="15" t="s">
-        <v>26</v>
-      </c>
-      <c r="I52" s="16"/>
-      <c r="J52" s="14"/>
-    </row>
-    <row r="53" spans="7:10" x14ac:dyDescent="0.3">
-      <c r="G53" s="10" t="s">
+      <c r="H56" s="15" t="s">
+        <v>29</v>
+      </c>
+      <c r="I56" s="16"/>
+      <c r="J56" s="14"/>
+    </row>
+    <row r="57" spans="7:10" x14ac:dyDescent="0.3">
+      <c r="G57" s="10" t="s">
         <v>14</v>
       </c>
-      <c r="H53" s="15" t="str">
-        <f>G51 &amp; "." &amp; H51 &amp; "-" &amp; H52</f>
-        <v>v10.0.2-Classic_Reimagined_10s</v>
-      </c>
-      <c r="I53" s="16"/>
-      <c r="J53" s="14"/>
-    </row>
-    <row r="54" spans="7:10" x14ac:dyDescent="0.3">
-      <c r="G54" s="10" t="s">
-        <v>15</v>
-      </c>
-      <c r="H54" s="15" t="str">
-        <f>H53 &amp; "-build-" &amp; I51</f>
-        <v>v10.0.2-Classic_Reimagined_10s-build-6309-rt6</v>
-      </c>
-      <c r="I54" s="16"/>
-    </row>
-    <row r="55" spans="7:10" x14ac:dyDescent="0.3">
-      <c r="G55" s="7" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="56" spans="7:10" x14ac:dyDescent="0.3">
-      <c r="G56" s="8" t="s">
-        <v>17</v>
-      </c>
-      <c r="H56" s="8" t="s">
-        <v>6</v>
-      </c>
-      <c r="I56" s="8" t="s">
-        <v>3</v>
-      </c>
-      <c r="J56" s="8" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="57" spans="7:10" x14ac:dyDescent="0.3">
-      <c r="G57" s="9" t="s">
-        <v>11</v>
-      </c>
-      <c r="H57" s="9">
-        <v>1</v>
-      </c>
-      <c r="I57" s="9" t="str">
-        <f>I51</f>
-        <v>6309-rt6</v>
-      </c>
-      <c r="J57" s="9" t="s">
-        <v>28</v>
-      </c>
+      <c r="H57" s="15" t="str">
+        <f>G55 &amp; "." &amp; H55 &amp; "-" &amp; H56</f>
+        <v>v10.0.1-Classic_Reimagined_10</v>
+      </c>
+      <c r="I57" s="16"/>
+      <c r="J57" s="14"/>
     </row>
     <row r="58" spans="7:10" x14ac:dyDescent="0.3">
       <c r="G58" s="10" t="s">
+        <v>15</v>
+      </c>
+      <c r="H58" s="15" t="str">
+        <f>H57 &amp; "-build-" &amp; I55</f>
+        <v>v10.0.1-Classic_Reimagined_10-build-6309-rt6</v>
+      </c>
+      <c r="I58" s="16"/>
+    </row>
+    <row r="59" spans="7:10" x14ac:dyDescent="0.3">
+      <c r="G59" s="26" t="s">
+        <v>30</v>
+      </c>
+      <c r="H59" s="26"/>
+      <c r="I59" s="26"/>
+      <c r="J59" s="26"/>
+    </row>
+    <row r="60" spans="7:10" x14ac:dyDescent="0.3">
+      <c r="G60" s="7" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="61" spans="7:10" x14ac:dyDescent="0.3">
+      <c r="G61" s="8" t="s">
+        <v>17</v>
+      </c>
+      <c r="H61" s="8" t="s">
+        <v>6</v>
+      </c>
+      <c r="I61" s="8" t="s">
+        <v>3</v>
+      </c>
+      <c r="J61" s="8" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="62" spans="7:10" x14ac:dyDescent="0.3">
+      <c r="G62" s="9" t="s">
+        <v>32</v>
+      </c>
+      <c r="H62" s="9">
+        <v>32</v>
+      </c>
+      <c r="I62" s="9" t="str">
+        <f>I55</f>
+        <v>6309-rt6</v>
+      </c>
+      <c r="J62" s="9" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="63" spans="7:10" x14ac:dyDescent="0.3">
+      <c r="G63" s="10" t="s">
         <v>13</v>
       </c>
-      <c r="H58" s="15" t="s">
-        <v>29</v>
-      </c>
-      <c r="I58" s="16"/>
-      <c r="J58" s="14"/>
-    </row>
-    <row r="59" spans="7:10" x14ac:dyDescent="0.3">
-      <c r="G59" s="10" t="s">
+      <c r="H63" s="15" t="s">
+        <v>34</v>
+      </c>
+      <c r="I63" s="16"/>
+      <c r="J63" s="14"/>
+    </row>
+    <row r="64" spans="7:10" x14ac:dyDescent="0.3">
+      <c r="G64" s="10" t="s">
         <v>14</v>
       </c>
-      <c r="H59" s="15" t="str">
-        <f>G57 &amp; "." &amp; H57 &amp; "-" &amp; H58</f>
-        <v>v10.0.1-Classic_Reimagined_10</v>
-      </c>
-      <c r="I59" s="16"/>
-      <c r="J59" s="14"/>
-    </row>
-    <row r="60" spans="7:10" x14ac:dyDescent="0.3">
-      <c r="G60" s="10" t="s">
-        <v>15</v>
-      </c>
-      <c r="H60" s="15" t="str">
-        <f>H59 &amp; "-build-" &amp; I57</f>
-        <v>v10.0.1-Classic_Reimagined_10-build-6309-rt6</v>
-      </c>
-      <c r="I60" s="16"/>
-    </row>
-    <row r="61" spans="7:10" x14ac:dyDescent="0.3">
-      <c r="G61" s="43" t="s">
-        <v>30</v>
-      </c>
-      <c r="H61" s="43"/>
-      <c r="I61" s="43"/>
-      <c r="J61" s="43"/>
-    </row>
-    <row r="62" spans="7:10" x14ac:dyDescent="0.3">
-      <c r="G62" s="7" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="63" spans="7:10" x14ac:dyDescent="0.3">
-      <c r="G63" s="8" t="s">
-        <v>17</v>
-      </c>
-      <c r="H63" s="8" t="s">
-        <v>6</v>
-      </c>
-      <c r="I63" s="8" t="s">
-        <v>3</v>
-      </c>
-      <c r="J63" s="8" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="64" spans="7:10" x14ac:dyDescent="0.3">
-      <c r="G64" s="9" t="s">
-        <v>32</v>
-      </c>
-      <c r="H64" s="9">
-        <v>32</v>
-      </c>
-      <c r="I64" s="9" t="str">
-        <f>I57</f>
-        <v>6309-rt6</v>
-      </c>
-      <c r="J64" s="9" t="s">
-        <v>33</v>
-      </c>
+      <c r="H64" s="15" t="str">
+        <f>G62 &amp; "." &amp; H62 &amp; "-" &amp; H63</f>
+        <v>v8.10.32-Classic_Reimagined_8</v>
+      </c>
+      <c r="I64" s="16"/>
+      <c r="J64" s="14"/>
     </row>
     <row r="65" spans="7:10" x14ac:dyDescent="0.3">
       <c r="G65" s="10" t="s">
+        <v>15</v>
+      </c>
+      <c r="H65" s="15" t="str">
+        <f>H64 &amp; "-build-" &amp; I62</f>
+        <v>v8.10.32-Classic_Reimagined_8-build-6309-rt6</v>
+      </c>
+      <c r="I65" s="16"/>
+    </row>
+    <row r="66" spans="7:10" x14ac:dyDescent="0.3">
+      <c r="G66" s="7" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="67" spans="7:10" x14ac:dyDescent="0.3">
+      <c r="G67" s="8" t="s">
+        <v>17</v>
+      </c>
+      <c r="H67" s="8" t="s">
+        <v>6</v>
+      </c>
+      <c r="I67" s="8" t="s">
+        <v>3</v>
+      </c>
+      <c r="J67" s="8" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="68" spans="7:10" x14ac:dyDescent="0.3">
+      <c r="G68" s="9" t="s">
+        <v>32</v>
+      </c>
+      <c r="H68" s="9">
+        <v>31</v>
+      </c>
+      <c r="I68" s="9" t="str">
+        <f>I62</f>
+        <v>6309-rt6</v>
+      </c>
+      <c r="J68" s="9" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="69" spans="7:10" x14ac:dyDescent="0.3">
+      <c r="G69" s="10" t="s">
         <v>13</v>
       </c>
-      <c r="H65" s="15" t="s">
+      <c r="H69" s="15" t="s">
         <v>34</v>
       </c>
-      <c r="I65" s="16"/>
-      <c r="J65" s="14"/>
-    </row>
-    <row r="66" spans="7:10" x14ac:dyDescent="0.3">
-      <c r="G66" s="10" t="s">
+      <c r="I69" s="16"/>
+      <c r="J69" s="14"/>
+    </row>
+    <row r="70" spans="7:10" x14ac:dyDescent="0.3">
+      <c r="G70" s="10" t="s">
         <v>14</v>
       </c>
-      <c r="H66" s="15" t="str">
-        <f>G64 &amp; "." &amp; H64 &amp; "-" &amp; H65</f>
-        <v>v8.10.32-Classic_Reimagined_8</v>
-      </c>
-      <c r="I66" s="16"/>
-      <c r="J66" s="14"/>
-    </row>
-    <row r="67" spans="7:10" x14ac:dyDescent="0.3">
-      <c r="G67" s="10" t="s">
-        <v>15</v>
-      </c>
-      <c r="H67" s="15" t="str">
-        <f>H66 &amp; "-build-" &amp; I64</f>
-        <v>v8.10.32-Classic_Reimagined_8-build-6309-rt6</v>
-      </c>
-      <c r="I67" s="16"/>
-    </row>
-    <row r="68" spans="7:10" x14ac:dyDescent="0.3">
-      <c r="G68" s="7" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="69" spans="7:10" x14ac:dyDescent="0.3">
-      <c r="G69" s="8" t="s">
-        <v>17</v>
-      </c>
-      <c r="H69" s="8" t="s">
-        <v>6</v>
-      </c>
-      <c r="I69" s="8" t="s">
-        <v>3</v>
-      </c>
-      <c r="J69" s="8" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="70" spans="7:10" x14ac:dyDescent="0.3">
-      <c r="G70" s="9" t="s">
-        <v>32</v>
-      </c>
-      <c r="H70" s="9">
-        <v>31</v>
-      </c>
-      <c r="I70" s="9" t="str">
-        <f>I64</f>
-        <v>6309-rt6</v>
-      </c>
-      <c r="J70" s="9" t="s">
-        <v>35</v>
-      </c>
+      <c r="H70" s="15" t="str">
+        <f>G68 &amp; "." &amp; H68 &amp; "-" &amp; H69</f>
+        <v>v8.10.31-Classic_Reimagined_8</v>
+      </c>
+      <c r="I70" s="16"/>
+      <c r="J70" s="14"/>
     </row>
     <row r="71" spans="7:10" x14ac:dyDescent="0.3">
       <c r="G71" s="10" t="s">
+        <v>15</v>
+      </c>
+      <c r="H71" s="15" t="str">
+        <f>H70 &amp; "-build-" &amp; I68</f>
+        <v>v8.10.31-Classic_Reimagined_8-build-6309-rt6</v>
+      </c>
+      <c r="I71" s="16"/>
+    </row>
+    <row r="72" spans="7:10" x14ac:dyDescent="0.3">
+      <c r="G72" s="24" t="s">
+        <v>36</v>
+      </c>
+      <c r="H72" s="24"/>
+      <c r="I72" s="24"/>
+      <c r="J72" s="24"/>
+    </row>
+    <row r="73" spans="7:10" x14ac:dyDescent="0.3">
+      <c r="G73" s="8" t="s">
+        <v>17</v>
+      </c>
+      <c r="H73" s="8" t="s">
+        <v>6</v>
+      </c>
+      <c r="I73" s="8" t="s">
+        <v>3</v>
+      </c>
+      <c r="J73" s="8" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="74" spans="7:10" x14ac:dyDescent="0.3">
+      <c r="G74" s="9" t="s">
+        <v>37</v>
+      </c>
+      <c r="H74" s="9">
+        <v>3</v>
+      </c>
+      <c r="I74" s="9" t="str">
+        <f>I68</f>
+        <v>6309-rt6</v>
+      </c>
+      <c r="J74" s="9" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="75" spans="7:10" x14ac:dyDescent="0.3">
+      <c r="G75" s="10" t="s">
         <v>13</v>
       </c>
-      <c r="H71" s="15" t="s">
-        <v>34</v>
-      </c>
-      <c r="I71" s="16"/>
-      <c r="J71" s="14"/>
-    </row>
-    <row r="72" spans="7:10" x14ac:dyDescent="0.3">
-      <c r="G72" s="10" t="s">
+      <c r="H75" s="15" t="s">
+        <v>39</v>
+      </c>
+      <c r="I75" s="16"/>
+      <c r="J75" s="14"/>
+    </row>
+    <row r="76" spans="7:10" x14ac:dyDescent="0.3">
+      <c r="G76" s="10" t="s">
         <v>14</v>
       </c>
-      <c r="H72" s="15" t="str">
-        <f>G70 &amp; "." &amp; H70 &amp; "-" &amp; H71</f>
-        <v>v8.10.31-Classic_Reimagined_8</v>
-      </c>
-      <c r="I72" s="16"/>
-      <c r="J72" s="14"/>
-    </row>
-    <row r="73" spans="7:10" x14ac:dyDescent="0.3">
-      <c r="G73" s="10" t="s">
-        <v>15</v>
-      </c>
-      <c r="H73" s="15" t="str">
-        <f>H72 &amp; "-build-" &amp; I70</f>
-        <v>v8.10.31-Classic_Reimagined_8-build-6309-rt6</v>
-      </c>
-      <c r="I73" s="16"/>
-    </row>
-    <row r="74" spans="7:10" x14ac:dyDescent="0.3">
-      <c r="G74" s="44" t="s">
-        <v>36</v>
-      </c>
-      <c r="H74" s="44"/>
-      <c r="I74" s="44"/>
-      <c r="J74" s="44"/>
-    </row>
-    <row r="75" spans="7:10" x14ac:dyDescent="0.3">
-      <c r="G75" s="8" t="s">
-        <v>17</v>
-      </c>
-      <c r="H75" s="8" t="s">
-        <v>6</v>
-      </c>
-      <c r="I75" s="8" t="s">
-        <v>3</v>
-      </c>
-      <c r="J75" s="8" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="76" spans="7:10" x14ac:dyDescent="0.3">
-      <c r="G76" s="9" t="s">
-        <v>37</v>
-      </c>
-      <c r="H76" s="9">
-        <v>3</v>
-      </c>
-      <c r="I76" s="9" t="str">
-        <f>I70</f>
-        <v>6309-rt6</v>
-      </c>
-      <c r="J76" s="9" t="s">
-        <v>38</v>
-      </c>
+      <c r="H76" s="15" t="str">
+        <f>G74 &amp; "." &amp; H74 &amp; "-" &amp; H75</f>
+        <v>v7.11.3-Better_Default_7</v>
+      </c>
+      <c r="I76" s="16"/>
+      <c r="J76" s="14"/>
     </row>
     <row r="77" spans="7:10" x14ac:dyDescent="0.3">
       <c r="G77" s="10" t="s">
-        <v>13</v>
-      </c>
-      <c r="H77" s="15" t="s">
-        <v>39</v>
+        <v>15</v>
+      </c>
+      <c r="H77" s="15" t="str">
+        <f>H76 &amp; "-build-" &amp; I74</f>
+        <v>v7.11.3-Better_Default_7-build-6309-rt6</v>
       </c>
       <c r="I77" s="16"/>
-      <c r="J77" s="14"/>
-    </row>
-    <row r="78" spans="7:10" x14ac:dyDescent="0.3">
-      <c r="G78" s="10" t="s">
-        <v>14</v>
-      </c>
-      <c r="H78" s="15" t="str">
-        <f>G76 &amp; "." &amp; H76 &amp; "-" &amp; H77</f>
-        <v>v7.11.3-Better_Default_7</v>
-      </c>
-      <c r="I78" s="16"/>
-      <c r="J78" s="14"/>
-    </row>
-    <row r="79" spans="7:10" x14ac:dyDescent="0.3">
-      <c r="G79" s="10" t="s">
-        <v>15</v>
-      </c>
-      <c r="H79" s="15" t="str">
-        <f>H78 &amp; "-build-" &amp; I76</f>
-        <v>v7.11.3-Better_Default_7-build-6309-rt6</v>
-      </c>
-      <c r="I79" s="16"/>
     </row>
   </sheetData>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A10:A20">
     <sortCondition ref="A20"/>
   </sortState>
-  <mergeCells count="10">
-    <mergeCell ref="G74:J74"/>
-    <mergeCell ref="G1:K1"/>
-    <mergeCell ref="G15:K15"/>
-    <mergeCell ref="G61:J61"/>
-    <mergeCell ref="G8:K8"/>
+  <mergeCells count="9">
     <mergeCell ref="A1:E1"/>
     <mergeCell ref="C9:E9"/>
     <mergeCell ref="C10:E10"/>
     <mergeCell ref="A7:C7"/>
     <mergeCell ref="A8:C8"/>
+    <mergeCell ref="G1:K1"/>
+    <mergeCell ref="G13:K13"/>
+    <mergeCell ref="G59:J59"/>
+    <mergeCell ref="G72:J72"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
@@ -1777,12 +1762,12 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
-      <c r="A1" s="41" t="s">
+      <c r="A1" s="44" t="s">
         <v>40</v>
       </c>
-      <c r="B1" s="41"/>
-      <c r="C1" s="41"/>
-      <c r="D1" s="41"/>
+      <c r="B1" s="44"/>
+      <c r="C1" s="44"/>
+      <c r="D1" s="44"/>
     </row>
     <row r="2" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
@@ -1821,21 +1806,21 @@
       <c r="A5" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="B5" s="39" t="s">
+      <c r="B5" s="42" t="s">
         <v>45</v>
       </c>
-      <c r="C5" s="40"/>
+      <c r="C5" s="43"/>
       <c r="D5" s="5"/>
     </row>
     <row r="6" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A6" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="B6" s="39" t="str">
+      <c r="B6" s="42" t="str">
         <f>A4 &amp; "." &amp; B4 &amp; "." &amp; C4 &amp; "-" &amp; B5</f>
         <v>v6.0.7-Better_Default_6</v>
       </c>
-      <c r="C6" s="40"/>
+      <c r="C6" s="43"/>
       <c r="D6" s="5"/>
     </row>
     <row r="7" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
@@ -1875,21 +1860,21 @@
       <c r="A10" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="B10" s="39" t="s">
+      <c r="B10" s="42" t="s">
         <v>49</v>
       </c>
-      <c r="C10" s="40"/>
+      <c r="C10" s="43"/>
       <c r="D10" s="5"/>
     </row>
     <row r="11" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A11" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="B11" s="39" t="str">
+      <c r="B11" s="42" t="str">
         <f>A9 &amp; "." &amp; B9 &amp; "." &amp; C9 &amp; "-" &amp; B10</f>
         <v>v1.4.0-Better_Default_5</v>
       </c>
-      <c r="C11" s="40"/>
+      <c r="C11" s="43"/>
       <c r="D11" s="5"/>
     </row>
     <row r="12" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
@@ -1929,21 +1914,21 @@
       <c r="A15" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="B15" s="39" t="s">
+      <c r="B15" s="42" t="s">
         <v>52</v>
       </c>
-      <c r="C15" s="40"/>
+      <c r="C15" s="43"/>
       <c r="D15" s="5"/>
     </row>
     <row r="16" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A16" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="B16" s="39" t="str">
+      <c r="B16" s="42" t="str">
         <f>A14 &amp; "." &amp; B14 &amp; "." &amp; C14 &amp; "-" &amp; B15</f>
         <v>v1.3.0-Better_Default_4</v>
       </c>
-      <c r="C16" s="40"/>
+      <c r="C16" s="43"/>
       <c r="D16" s="5"/>
     </row>
     <row r="17" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
@@ -1983,21 +1968,21 @@
       <c r="A20" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="B20" s="39" t="s">
+      <c r="B20" s="42" t="s">
         <v>55</v>
       </c>
-      <c r="C20" s="40"/>
+      <c r="C20" s="43"/>
       <c r="D20" s="5"/>
     </row>
     <row r="21" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A21" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="B21" s="39" t="str">
+      <c r="B21" s="42" t="str">
         <f>A19 &amp; "." &amp; B19 &amp; "." &amp; C19 &amp; "-" &amp; B20</f>
         <v>v1.2.2-Better_Default_3.1</v>
       </c>
-      <c r="C21" s="40"/>
+      <c r="C21" s="43"/>
       <c r="D21" s="5"/>
     </row>
     <row r="22" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
@@ -2037,21 +2022,21 @@
       <c r="A25" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="B25" s="39" t="s">
+      <c r="B25" s="42" t="s">
         <v>56</v>
       </c>
-      <c r="C25" s="40"/>
+      <c r="C25" s="43"/>
       <c r="D25" s="5"/>
     </row>
     <row r="26" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A26" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="B26" s="39" t="str">
+      <c r="B26" s="42" t="str">
         <f>A24 &amp; "." &amp; B24 &amp; "." &amp; C24 &amp; "-" &amp; B25</f>
         <v>v1.2.1-Better_Default_3</v>
       </c>
-      <c r="C26" s="40"/>
+      <c r="C26" s="43"/>
       <c r="D26" s="5"/>
     </row>
     <row r="27" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
@@ -2091,21 +2076,21 @@
       <c r="A30" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="B30" s="39" t="s">
+      <c r="B30" s="42" t="s">
         <v>58</v>
       </c>
-      <c r="C30" s="40"/>
+      <c r="C30" s="43"/>
       <c r="D30" s="5"/>
     </row>
     <row r="31" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A31" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="B31" s="39" t="str">
+      <c r="B31" s="42" t="str">
         <f>A29 &amp; "." &amp; B29 &amp; "." &amp; C29 &amp; "-" &amp; B30</f>
         <v>v1.2.0-Better_Default_2</v>
       </c>
-      <c r="C31" s="40"/>
+      <c r="C31" s="43"/>
       <c r="D31" s="5"/>
     </row>
     <row r="32" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
@@ -2145,21 +2130,21 @@
       <c r="A35" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="B35" s="39" t="s">
+      <c r="B35" s="42" t="s">
         <v>60</v>
       </c>
-      <c r="C35" s="40"/>
+      <c r="C35" s="43"/>
       <c r="D35" s="5"/>
     </row>
     <row r="36" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A36" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="B36" s="39" t="str">
+      <c r="B36" s="42" t="str">
         <f>A34 &amp; "." &amp; B34 &amp; "." &amp; C34 &amp; "-" &amp; B35</f>
         <v>v1.1.1-Better_Default</v>
       </c>
-      <c r="C36" s="40"/>
+      <c r="C36" s="43"/>
       <c r="D36" s="5"/>
     </row>
     <row r="37" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
@@ -2199,30 +2184,25 @@
       <c r="A40" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="B40" s="39" t="s">
+      <c r="B40" s="42" t="s">
         <v>60</v>
       </c>
-      <c r="C40" s="40"/>
+      <c r="C40" s="43"/>
       <c r="D40" s="5"/>
     </row>
     <row r="41" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A41" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="B41" s="39" t="str">
+      <c r="B41" s="42" t="str">
         <f>A39 &amp; "." &amp; B39 &amp; "." &amp; C39 &amp; "-" &amp; B40</f>
         <v>v1.1.0-Better_Default</v>
       </c>
-      <c r="C41" s="40"/>
+      <c r="C41" s="43"/>
       <c r="D41" s="5"/>
     </row>
   </sheetData>
   <mergeCells count="17">
-    <mergeCell ref="B41:C41"/>
-    <mergeCell ref="B36:C36"/>
-    <mergeCell ref="B35:C35"/>
-    <mergeCell ref="B31:C31"/>
-    <mergeCell ref="B30:C30"/>
     <mergeCell ref="B10:C10"/>
     <mergeCell ref="B6:C6"/>
     <mergeCell ref="B5:C5"/>
@@ -2235,6 +2215,11 @@
     <mergeCell ref="B16:C16"/>
     <mergeCell ref="B15:C15"/>
     <mergeCell ref="B11:C11"/>
+    <mergeCell ref="B41:C41"/>
+    <mergeCell ref="B36:C36"/>
+    <mergeCell ref="B35:C35"/>
+    <mergeCell ref="B31:C31"/>
+    <mergeCell ref="B30:C30"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait"/>

</xml_diff>

<commit_message>
Added 26.4 shader compatibility
Adds a new 26.4 shader pack with updated cloud, lightmap, terrain, fog, and texture sampling shaders for newer Minecraft shader formats. This also refreshes the existing 26.3 cloud shader to the newer GLSL version and updates the pack metadata to register the new compatibility range.
</commit_message>
<xml_diff>
--- a/version_guide.xlsx
+++ b/version_guide.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\PrismLauncher\instances\NeoBeta Remastered\minecraft\resourcepacks\Classic-Reimagined\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{94A079A0-5E8A-4040-A3C2-16E0F54F821A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3651B3C6-EED2-4052-AD8F-02A711BE96CF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="521" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="233" uniqueCount="78">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="243" uniqueCount="79">
   <si>
     <t>Current version in development</t>
   </si>
@@ -268,6 +268,9 @@
   </si>
   <si>
     <t>Fixed baby rabbit model</t>
+  </si>
+  <si>
+    <t>Added 26.4 shader compatibility</t>
   </si>
 </sst>
 </file>
@@ -760,7 +763,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:K77"/>
+  <dimension ref="A1:K82"/>
   <sheetFormatPr defaultColWidth="27.28515625" defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="36.5703125" style="6" customWidth="1"/>
@@ -800,7 +803,7 @@
         <v>64</v>
       </c>
       <c r="B3" s="22">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G3" s="8" t="s">
         <v>2</v>
@@ -823,7 +826,7 @@
         <v>63</v>
       </c>
       <c r="B4" s="22">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="G4" s="9" t="s">
         <v>11</v>
@@ -832,11 +835,11 @@
         <v>11</v>
       </c>
       <c r="I4" s="9">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="J4" s="9" t="str">
         <f>D8</f>
-        <v>6309-rt6</v>
+        <v>6410-rt6</v>
       </c>
       <c r="K4" s="9">
         <v>26.3</v>
@@ -866,14 +869,14 @@
       </c>
       <c r="B6" s="23">
         <f>(B2*1000)+(B3*100)+B4+((B5-2026)*1000)</f>
-        <v>6309</v>
+        <v>6410</v>
       </c>
       <c r="G6" s="10" t="s">
         <v>14</v>
       </c>
       <c r="H6" s="11" t="str">
         <f>G4 &amp; "." &amp; H4 &amp; "_" &amp; I4 &amp; "-" &amp; H5</f>
-        <v>v10.0.11_3-DogePack_Classic_11_Beta</v>
+        <v>v10.0.11_4-DogePack_Classic_11_Beta</v>
       </c>
       <c r="I6" s="12"/>
       <c r="J6" s="13"/>
@@ -896,7 +899,7 @@
       </c>
       <c r="H7" s="11" t="str">
         <f>H6 &amp; "-build-" &amp; J4</f>
-        <v>v10.0.11_3-DogePack_Classic_11_Beta-build-6309-rt6</v>
+        <v>v10.0.11_4-DogePack_Classic_11_Beta-build-6410-rt6</v>
       </c>
       <c r="I7" s="12"/>
       <c r="J7" s="13"/>
@@ -904,16 +907,16 @@
     <row r="8" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A8" s="39" t="str">
         <f>G4 &amp; "." &amp; H4 &amp; "_" &amp; I4 &amp; "-build-" &amp; D8</f>
-        <v>v10.0.11_3-build-6309-rt6</v>
+        <v>v10.0.11_4-build-6410-rt6</v>
       </c>
       <c r="B8" s="40"/>
       <c r="C8" s="41"/>
       <c r="D8" s="9" t="str">
         <f>B6&amp;"-rt"&amp;B2</f>
-        <v>6309-rt6</v>
+        <v>6410-rt6</v>
       </c>
       <c r="E8" s="18">
-        <f>K9</f>
+        <f>K14</f>
         <v>26.3</v>
       </c>
       <c r="G8" s="8" t="s">
@@ -951,11 +954,11 @@
         <v>11</v>
       </c>
       <c r="I9" s="9">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="J9" s="9" t="str">
         <f>J4</f>
-        <v>6309-rt6</v>
+        <v>6410-rt6</v>
       </c>
       <c r="K9" s="9">
         <v>26.3</v>
@@ -974,8 +977,8 @@
         <v>13</v>
       </c>
       <c r="H10" s="11" t="str">
-        <f>H5</f>
-        <v>DogePack_Classic_11_Beta</v>
+        <f>"DogePack_Classic" &amp; G7</f>
+        <v>DogePack_ClassicResource Pack Build</v>
       </c>
       <c r="I10" s="12"/>
       <c r="J10" s="13"/>
@@ -990,7 +993,7 @@
       </c>
       <c r="H11" s="11" t="str">
         <f>G9 &amp; "." &amp; H9 &amp; "_" &amp; I9 &amp; "-" &amp; H10</f>
-        <v>v10.0.11_2-DogePack_Classic_11_Beta</v>
+        <v>v10.0.11_3-DogePack_ClassicResource Pack Build</v>
       </c>
       <c r="I11" s="12"/>
       <c r="J11" s="13"/>
@@ -1005,7 +1008,7 @@
       </c>
       <c r="H12" s="11" t="str">
         <f>H11 &amp; "-build-" &amp; J9</f>
-        <v>v10.0.11_2-DogePack_Classic_11_Beta-build-6309-rt6</v>
+        <v>v10.0.11_3-DogePack_ClassicResource Pack Build-build-6410-rt6</v>
       </c>
       <c r="I12" s="12"/>
       <c r="J12" s="13"/>
@@ -1014,169 +1017,181 @@
       <c r="A13" s="6" t="s">
         <v>72</v>
       </c>
-      <c r="G13" s="25" t="s">
-        <v>1</v>
-      </c>
-      <c r="H13" s="25"/>
-      <c r="I13" s="25"/>
-      <c r="J13" s="25"/>
-      <c r="K13" s="25"/>
+      <c r="G13" s="8" t="s">
+        <v>2</v>
+      </c>
+      <c r="H13" s="8" t="s">
+        <v>6</v>
+      </c>
+      <c r="I13" s="8" t="s">
+        <v>7</v>
+      </c>
+      <c r="J13" s="8" t="s">
+        <v>3</v>
+      </c>
+      <c r="K13" s="8" t="s">
+        <v>4</v>
+      </c>
     </row>
     <row r="14" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A14" s="6" t="s">
         <v>73</v>
       </c>
-      <c r="G14" s="7" t="s">
-        <v>5</v>
+      <c r="G14" s="9" t="s">
+        <v>11</v>
+      </c>
+      <c r="H14" s="9">
+        <v>11</v>
+      </c>
+      <c r="I14" s="9">
+        <v>2</v>
+      </c>
+      <c r="J14" s="9" t="str">
+        <f>J9</f>
+        <v>6410-rt6</v>
+      </c>
+      <c r="K14" s="9">
+        <v>26.3</v>
       </c>
     </row>
     <row r="15" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A15" s="6" t="s">
         <v>74</v>
       </c>
-      <c r="G15" s="8" t="s">
-        <v>2</v>
-      </c>
-      <c r="H15" s="8" t="s">
-        <v>6</v>
-      </c>
-      <c r="I15" s="8" t="s">
-        <v>7</v>
-      </c>
-      <c r="J15" s="8" t="s">
-        <v>3</v>
-      </c>
-      <c r="K15" s="8" t="s">
-        <v>4</v>
-      </c>
+      <c r="G15" s="10" t="s">
+        <v>13</v>
+      </c>
+      <c r="H15" s="11" t="str">
+        <f>H5</f>
+        <v>DogePack_Classic_11_Beta</v>
+      </c>
+      <c r="I15" s="12"/>
+      <c r="J15" s="13"/>
+      <c r="K15" s="14"/>
     </row>
     <row r="16" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A16" s="6" t="s">
         <v>75</v>
       </c>
-      <c r="G16" s="9" t="s">
-        <v>11</v>
-      </c>
-      <c r="H16" s="9">
-        <v>11</v>
-      </c>
-      <c r="I16" s="9">
-        <v>1</v>
-      </c>
-      <c r="J16" s="9" t="str">
-        <f>J9</f>
-        <v>6309-rt6</v>
-      </c>
-      <c r="K16" s="9">
-        <v>26.1</v>
-      </c>
+      <c r="G16" s="10" t="s">
+        <v>14</v>
+      </c>
+      <c r="H16" s="11" t="str">
+        <f>G14 &amp; "." &amp; H14 &amp; "_" &amp; I14 &amp; "-" &amp; H15</f>
+        <v>v10.0.11_2-DogePack_Classic_11_Beta</v>
+      </c>
+      <c r="I16" s="12"/>
+      <c r="J16" s="13"/>
+      <c r="K16" s="14"/>
     </row>
     <row r="17" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A17" s="6" t="s">
         <v>76</v>
       </c>
       <c r="G17" s="10" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="H17" s="11" t="str">
-        <f>"Classic_Reimagined_10" &amp; G14</f>
-        <v>Classic_Reimagined_10_SE_2.1</v>
+        <f>H16 &amp; "-build-" &amp; J14</f>
+        <v>v10.0.11_2-DogePack_Classic_11_Beta-build-6410-rt6</v>
       </c>
       <c r="I17" s="12"/>
       <c r="J17" s="13"/>
-      <c r="K17" s="14"/>
     </row>
     <row r="18" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A18" s="6" t="s">
         <v>77</v>
       </c>
-      <c r="G18" s="10" t="s">
-        <v>14</v>
-      </c>
-      <c r="H18" s="11" t="str">
-        <f>G16 &amp; "." &amp; H16 &amp; "_" &amp; I16 &amp; "-" &amp; H17</f>
-        <v>v10.0.11_1-Classic_Reimagined_10_SE_2.1</v>
-      </c>
-      <c r="I18" s="12"/>
-      <c r="J18" s="13"/>
-      <c r="K18" s="14"/>
+      <c r="G18" s="25" t="s">
+        <v>1</v>
+      </c>
+      <c r="H18" s="25"/>
+      <c r="I18" s="25"/>
+      <c r="J18" s="25"/>
+      <c r="K18" s="25"/>
     </row>
     <row r="19" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="G19" s="10" t="s">
-        <v>15</v>
-      </c>
-      <c r="H19" s="11" t="str">
-        <f>H18 &amp; "-build-" &amp; J16</f>
-        <v>v10.0.11_1-Classic_Reimagined_10_SE_2.1-build-6309-rt6</v>
-      </c>
-      <c r="I19" s="12"/>
-      <c r="J19" s="13"/>
+      <c r="A19" s="6" t="s">
+        <v>78</v>
+      </c>
+      <c r="G19" s="7" t="s">
+        <v>5</v>
+      </c>
     </row>
     <row r="20" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="G20" s="7" t="s">
-        <v>16</v>
+      <c r="G20" s="8" t="s">
+        <v>2</v>
+      </c>
+      <c r="H20" s="8" t="s">
+        <v>6</v>
+      </c>
+      <c r="I20" s="8" t="s">
+        <v>7</v>
+      </c>
+      <c r="J20" s="8" t="s">
+        <v>3</v>
+      </c>
+      <c r="K20" s="8" t="s">
+        <v>4</v>
       </c>
     </row>
     <row r="21" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="G21" s="8" t="s">
-        <v>17</v>
-      </c>
-      <c r="H21" s="8" t="s">
-        <v>6</v>
-      </c>
-      <c r="I21" s="8" t="s">
-        <v>3</v>
-      </c>
-      <c r="J21" s="8" t="s">
-        <v>4</v>
+      <c r="G21" s="9" t="s">
+        <v>11</v>
+      </c>
+      <c r="H21" s="9">
+        <v>11</v>
+      </c>
+      <c r="I21" s="9">
+        <v>1</v>
+      </c>
+      <c r="J21" s="9" t="str">
+        <f>J14</f>
+        <v>6410-rt6</v>
+      </c>
+      <c r="K21" s="9">
+        <v>26.1</v>
       </c>
     </row>
     <row r="22" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="G22" s="9" t="s">
-        <v>11</v>
-      </c>
-      <c r="H22" s="9">
-        <v>10</v>
-      </c>
-      <c r="I22" s="9" t="str">
-        <f>J16</f>
-        <v>6309-rt6</v>
-      </c>
-      <c r="J22" s="9" t="s">
-        <v>18</v>
-      </c>
+      <c r="G22" s="10" t="s">
+        <v>13</v>
+      </c>
+      <c r="H22" s="11" t="str">
+        <f>"Classic_Reimagined_10" &amp; G19</f>
+        <v>Classic_Reimagined_10_SE_2.1</v>
+      </c>
+      <c r="I22" s="12"/>
+      <c r="J22" s="13"/>
+      <c r="K22" s="14"/>
     </row>
     <row r="23" spans="1:11" x14ac:dyDescent="0.3">
       <c r="G23" s="10" t="s">
-        <v>13</v>
-      </c>
-      <c r="H23" s="15" t="str">
-        <f>"Classic_Reimagined_10" &amp; G20</f>
-        <v>Classic_Reimagined_10_SE_2</v>
-      </c>
-      <c r="I23" s="16"/>
-      <c r="J23" s="14"/>
+        <v>14</v>
+      </c>
+      <c r="H23" s="11" t="str">
+        <f>G21 &amp; "." &amp; H21 &amp; "_" &amp; I21 &amp; "-" &amp; H22</f>
+        <v>v10.0.11_1-Classic_Reimagined_10_SE_2.1</v>
+      </c>
+      <c r="I23" s="12"/>
+      <c r="J23" s="13"/>
+      <c r="K23" s="14"/>
     </row>
     <row r="24" spans="1:11" x14ac:dyDescent="0.3">
       <c r="G24" s="10" t="s">
-        <v>14</v>
-      </c>
-      <c r="H24" s="15" t="str">
-        <f>G22 &amp; "." &amp; H22 &amp; "-" &amp; H23</f>
-        <v>v10.0.10-Classic_Reimagined_10_SE_2</v>
-      </c>
-      <c r="I24" s="16"/>
-      <c r="J24" s="14"/>
+        <v>15</v>
+      </c>
+      <c r="H24" s="11" t="str">
+        <f>H23 &amp; "-build-" &amp; J21</f>
+        <v>v10.0.11_1-Classic_Reimagined_10_SE_2.1-build-6410-rt6</v>
+      </c>
+      <c r="I24" s="12"/>
+      <c r="J24" s="13"/>
     </row>
     <row r="25" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="G25" s="10" t="s">
-        <v>15</v>
-      </c>
-      <c r="H25" s="15" t="str">
-        <f>H24 &amp; "-build-" &amp; I22</f>
-        <v>v10.0.10-Classic_Reimagined_10_SE_2-build-6309-rt6</v>
-      </c>
-      <c r="I25" s="16"/>
+      <c r="G25" s="7" t="s">
+        <v>16</v>
+      </c>
     </row>
     <row r="26" spans="1:11" x14ac:dyDescent="0.3">
       <c r="G26" s="8" t="s">
@@ -1197,14 +1212,14 @@
         <v>11</v>
       </c>
       <c r="H27" s="9">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="I27" s="9" t="str">
-        <f>I22</f>
-        <v>6309-rt6</v>
+        <f>J21</f>
+        <v>6410-rt6</v>
       </c>
       <c r="J27" s="9" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="28" spans="1:11" x14ac:dyDescent="0.3">
@@ -1212,7 +1227,7 @@
         <v>13</v>
       </c>
       <c r="H28" s="15" t="str">
-        <f>H23</f>
+        <f>"Classic_Reimagined_10" &amp; G25</f>
         <v>Classic_Reimagined_10_SE_2</v>
       </c>
       <c r="I28" s="16"/>
@@ -1224,7 +1239,7 @@
       </c>
       <c r="H29" s="15" t="str">
         <f>G27 &amp; "." &amp; H27 &amp; "-" &amp; H28</f>
-        <v>v10.0.9-Classic_Reimagined_10_SE_2</v>
+        <v>v10.0.10-Classic_Reimagined_10_SE_2</v>
       </c>
       <c r="I29" s="16"/>
       <c r="J29" s="14"/>
@@ -1235,7 +1250,7 @@
       </c>
       <c r="H30" s="15" t="str">
         <f>H29 &amp; "-build-" &amp; I27</f>
-        <v>v10.0.9-Classic_Reimagined_10_SE_2-build-6309-rt6</v>
+        <v>v10.0.10-Classic_Reimagined_10_SE_2-build-6410-rt6</v>
       </c>
       <c r="I30" s="16"/>
     </row>
@@ -1258,14 +1273,14 @@
         <v>11</v>
       </c>
       <c r="H32" s="9">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="I32" s="9" t="str">
         <f>I27</f>
-        <v>6309-rt6</v>
+        <v>6410-rt6</v>
       </c>
       <c r="J32" s="9" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
     </row>
     <row r="33" spans="7:10" x14ac:dyDescent="0.3">
@@ -1285,7 +1300,7 @@
       </c>
       <c r="H34" s="15" t="str">
         <f>G32 &amp; "." &amp; H32 &amp; "-" &amp; H33</f>
-        <v>v10.0.7-Classic_Reimagined_10_SE_2</v>
+        <v>v10.0.9-Classic_Reimagined_10_SE_2</v>
       </c>
       <c r="I34" s="16"/>
       <c r="J34" s="14"/>
@@ -1296,7 +1311,7 @@
       </c>
       <c r="H35" s="15" t="str">
         <f>H34 &amp; "-build-" &amp; I32</f>
-        <v>v10.0.7-Classic_Reimagined_10_SE_2-build-6309-rt6</v>
+        <v>v10.0.9-Classic_Reimagined_10_SE_2-build-6410-rt6</v>
       </c>
       <c r="I35" s="16"/>
     </row>
@@ -1319,14 +1334,14 @@
         <v>11</v>
       </c>
       <c r="H37" s="9">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="I37" s="9" t="str">
         <f>I32</f>
-        <v>6309-rt6</v>
+        <v>6410-rt6</v>
       </c>
       <c r="J37" s="9" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="38" spans="7:10" x14ac:dyDescent="0.3">
@@ -1346,7 +1361,7 @@
       </c>
       <c r="H39" s="15" t="str">
         <f>G37 &amp; "." &amp; H37 &amp; "-" &amp; H38</f>
-        <v>v10.0.4-Classic_Reimagined_10_SE_2</v>
+        <v>v10.0.7-Classic_Reimagined_10_SE_2</v>
       </c>
       <c r="I39" s="16"/>
       <c r="J39" s="14"/>
@@ -1357,421 +1372,482 @@
       </c>
       <c r="H40" s="15" t="str">
         <f>H39 &amp; "-build-" &amp; I37</f>
-        <v>v10.0.4-Classic_Reimagined_10_SE_2-build-6309-rt6</v>
+        <v>v10.0.7-Classic_Reimagined_10_SE_2-build-6410-rt6</v>
       </c>
       <c r="I40" s="16"/>
     </row>
     <row r="41" spans="7:10" x14ac:dyDescent="0.3">
-      <c r="G41" s="7" t="s">
-        <v>22</v>
+      <c r="G41" s="8" t="s">
+        <v>17</v>
+      </c>
+      <c r="H41" s="8" t="s">
+        <v>6</v>
+      </c>
+      <c r="I41" s="8" t="s">
+        <v>3</v>
+      </c>
+      <c r="J41" s="8" t="s">
+        <v>4</v>
       </c>
     </row>
     <row r="42" spans="7:10" x14ac:dyDescent="0.3">
-      <c r="G42" s="8" t="s">
-        <v>17</v>
-      </c>
-      <c r="H42" s="8" t="s">
-        <v>6</v>
-      </c>
-      <c r="I42" s="8" t="s">
-        <v>3</v>
-      </c>
-      <c r="J42" s="8" t="s">
-        <v>4</v>
+      <c r="G42" s="9" t="s">
+        <v>11</v>
+      </c>
+      <c r="H42" s="9">
+        <v>4</v>
+      </c>
+      <c r="I42" s="9" t="str">
+        <f>I37</f>
+        <v>6410-rt6</v>
+      </c>
+      <c r="J42" s="9" t="s">
+        <v>21</v>
       </c>
     </row>
     <row r="43" spans="7:10" x14ac:dyDescent="0.3">
-      <c r="G43" s="9" t="s">
-        <v>11</v>
-      </c>
-      <c r="H43" s="9">
-        <v>3</v>
-      </c>
-      <c r="I43" s="9" t="str">
-        <f>I37</f>
-        <v>6309-rt6</v>
-      </c>
-      <c r="J43" s="9" t="s">
-        <v>23</v>
-      </c>
+      <c r="G43" s="10" t="s">
+        <v>13</v>
+      </c>
+      <c r="H43" s="15" t="str">
+        <f>H38</f>
+        <v>Classic_Reimagined_10_SE_2</v>
+      </c>
+      <c r="I43" s="16"/>
+      <c r="J43" s="14"/>
     </row>
     <row r="44" spans="7:10" x14ac:dyDescent="0.3">
       <c r="G44" s="10" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="H44" s="15" t="str">
-        <f>"Classic_Reimagined_10" &amp; G41</f>
-        <v>Classic_Reimagined_10_SE</v>
+        <f>G42 &amp; "." &amp; H42 &amp; "-" &amp; H43</f>
+        <v>v10.0.4-Classic_Reimagined_10_SE_2</v>
       </c>
       <c r="I44" s="16"/>
       <c r="J44" s="14"/>
     </row>
     <row r="45" spans="7:10" x14ac:dyDescent="0.3">
       <c r="G45" s="10" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="H45" s="15" t="str">
-        <f>G43 &amp; "." &amp; H43 &amp; "-" &amp; H44</f>
-        <v>v10.0.3-Classic_Reimagined_10_SE</v>
+        <f>H44 &amp; "-build-" &amp; I42</f>
+        <v>v10.0.4-Classic_Reimagined_10_SE_2-build-6410-rt6</v>
       </c>
       <c r="I45" s="16"/>
-      <c r="J45" s="14"/>
     </row>
     <row r="46" spans="7:10" x14ac:dyDescent="0.3">
-      <c r="G46" s="10" t="s">
-        <v>15</v>
-      </c>
-      <c r="H46" s="15" t="str">
-        <f>H45 &amp; "-build-" &amp; I43</f>
-        <v>v10.0.3-Classic_Reimagined_10_SE-build-6309-rt6</v>
-      </c>
-      <c r="I46" s="16"/>
+      <c r="G46" s="7" t="s">
+        <v>22</v>
+      </c>
     </row>
     <row r="47" spans="7:10" x14ac:dyDescent="0.3">
-      <c r="G47" s="7" t="s">
-        <v>24</v>
+      <c r="G47" s="8" t="s">
+        <v>17</v>
+      </c>
+      <c r="H47" s="8" t="s">
+        <v>6</v>
+      </c>
+      <c r="I47" s="8" t="s">
+        <v>3</v>
+      </c>
+      <c r="J47" s="8" t="s">
+        <v>4</v>
       </c>
     </row>
     <row r="48" spans="7:10" x14ac:dyDescent="0.3">
-      <c r="G48" s="8" t="s">
-        <v>17</v>
-      </c>
-      <c r="H48" s="8" t="s">
-        <v>6</v>
-      </c>
-      <c r="I48" s="8" t="s">
+      <c r="G48" s="9" t="s">
+        <v>11</v>
+      </c>
+      <c r="H48" s="9">
         <v>3</v>
       </c>
-      <c r="J48" s="8" t="s">
-        <v>4</v>
+      <c r="I48" s="9" t="str">
+        <f>I42</f>
+        <v>6410-rt6</v>
+      </c>
+      <c r="J48" s="9" t="s">
+        <v>23</v>
       </c>
     </row>
     <row r="49" spans="7:10" x14ac:dyDescent="0.3">
-      <c r="G49" s="9" t="s">
-        <v>11</v>
-      </c>
-      <c r="H49" s="9">
-        <v>2</v>
-      </c>
-      <c r="I49" s="9" t="str">
-        <f>I43</f>
-        <v>6309-rt6</v>
-      </c>
-      <c r="J49" s="9" t="s">
-        <v>25</v>
-      </c>
+      <c r="G49" s="10" t="s">
+        <v>13</v>
+      </c>
+      <c r="H49" s="15" t="str">
+        <f>"Classic_Reimagined_10" &amp; G46</f>
+        <v>Classic_Reimagined_10_SE</v>
+      </c>
+      <c r="I49" s="16"/>
+      <c r="J49" s="14"/>
     </row>
     <row r="50" spans="7:10" x14ac:dyDescent="0.3">
       <c r="G50" s="10" t="s">
-        <v>13</v>
-      </c>
-      <c r="H50" s="15" t="s">
-        <v>26</v>
+        <v>14</v>
+      </c>
+      <c r="H50" s="15" t="str">
+        <f>G48 &amp; "." &amp; H48 &amp; "-" &amp; H49</f>
+        <v>v10.0.3-Classic_Reimagined_10_SE</v>
       </c>
       <c r="I50" s="16"/>
       <c r="J50" s="14"/>
     </row>
     <row r="51" spans="7:10" x14ac:dyDescent="0.3">
       <c r="G51" s="10" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="H51" s="15" t="str">
-        <f>G49 &amp; "." &amp; H49 &amp; "-" &amp; H50</f>
-        <v>v10.0.2-Classic_Reimagined_10s</v>
+        <f>H50 &amp; "-build-" &amp; I48</f>
+        <v>v10.0.3-Classic_Reimagined_10_SE-build-6410-rt6</v>
       </c>
       <c r="I51" s="16"/>
-      <c r="J51" s="14"/>
     </row>
     <row r="52" spans="7:10" x14ac:dyDescent="0.3">
-      <c r="G52" s="10" t="s">
-        <v>15</v>
-      </c>
-      <c r="H52" s="15" t="str">
-        <f>H51 &amp; "-build-" &amp; I49</f>
-        <v>v10.0.2-Classic_Reimagined_10s-build-6309-rt6</v>
-      </c>
-      <c r="I52" s="16"/>
+      <c r="G52" s="7" t="s">
+        <v>24</v>
+      </c>
     </row>
     <row r="53" spans="7:10" x14ac:dyDescent="0.3">
-      <c r="G53" s="7" t="s">
-        <v>27</v>
+      <c r="G53" s="8" t="s">
+        <v>17</v>
+      </c>
+      <c r="H53" s="8" t="s">
+        <v>6</v>
+      </c>
+      <c r="I53" s="8" t="s">
+        <v>3</v>
+      </c>
+      <c r="J53" s="8" t="s">
+        <v>4</v>
       </c>
     </row>
     <row r="54" spans="7:10" x14ac:dyDescent="0.3">
-      <c r="G54" s="8" t="s">
-        <v>17</v>
-      </c>
-      <c r="H54" s="8" t="s">
-        <v>6</v>
-      </c>
-      <c r="I54" s="8" t="s">
-        <v>3</v>
-      </c>
-      <c r="J54" s="8" t="s">
-        <v>4</v>
+      <c r="G54" s="9" t="s">
+        <v>11</v>
+      </c>
+      <c r="H54" s="9">
+        <v>2</v>
+      </c>
+      <c r="I54" s="9" t="str">
+        <f>I48</f>
+        <v>6410-rt6</v>
+      </c>
+      <c r="J54" s="9" t="s">
+        <v>25</v>
       </c>
     </row>
     <row r="55" spans="7:10" x14ac:dyDescent="0.3">
-      <c r="G55" s="9" t="s">
-        <v>11</v>
-      </c>
-      <c r="H55" s="9">
-        <v>1</v>
-      </c>
-      <c r="I55" s="9" t="str">
-        <f>I49</f>
-        <v>6309-rt6</v>
-      </c>
-      <c r="J55" s="9" t="s">
-        <v>28</v>
-      </c>
+      <c r="G55" s="10" t="s">
+        <v>13</v>
+      </c>
+      <c r="H55" s="15" t="s">
+        <v>26</v>
+      </c>
+      <c r="I55" s="16"/>
+      <c r="J55" s="14"/>
     </row>
     <row r="56" spans="7:10" x14ac:dyDescent="0.3">
       <c r="G56" s="10" t="s">
-        <v>13</v>
-      </c>
-      <c r="H56" s="15" t="s">
-        <v>29</v>
+        <v>14</v>
+      </c>
+      <c r="H56" s="15" t="str">
+        <f>G54 &amp; "." &amp; H54 &amp; "-" &amp; H55</f>
+        <v>v10.0.2-Classic_Reimagined_10s</v>
       </c>
       <c r="I56" s="16"/>
       <c r="J56" s="14"/>
     </row>
     <row r="57" spans="7:10" x14ac:dyDescent="0.3">
       <c r="G57" s="10" t="s">
+        <v>15</v>
+      </c>
+      <c r="H57" s="15" t="str">
+        <f>H56 &amp; "-build-" &amp; I54</f>
+        <v>v10.0.2-Classic_Reimagined_10s-build-6410-rt6</v>
+      </c>
+      <c r="I57" s="16"/>
+    </row>
+    <row r="58" spans="7:10" x14ac:dyDescent="0.3">
+      <c r="G58" s="7" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="59" spans="7:10" x14ac:dyDescent="0.3">
+      <c r="G59" s="8" t="s">
+        <v>17</v>
+      </c>
+      <c r="H59" s="8" t="s">
+        <v>6</v>
+      </c>
+      <c r="I59" s="8" t="s">
+        <v>3</v>
+      </c>
+      <c r="J59" s="8" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="60" spans="7:10" x14ac:dyDescent="0.3">
+      <c r="G60" s="9" t="s">
+        <v>11</v>
+      </c>
+      <c r="H60" s="9">
+        <v>1</v>
+      </c>
+      <c r="I60" s="9" t="str">
+        <f>I54</f>
+        <v>6410-rt6</v>
+      </c>
+      <c r="J60" s="9" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="61" spans="7:10" x14ac:dyDescent="0.3">
+      <c r="G61" s="10" t="s">
+        <v>13</v>
+      </c>
+      <c r="H61" s="15" t="s">
+        <v>29</v>
+      </c>
+      <c r="I61" s="16"/>
+      <c r="J61" s="14"/>
+    </row>
+    <row r="62" spans="7:10" x14ac:dyDescent="0.3">
+      <c r="G62" s="10" t="s">
         <v>14</v>
       </c>
-      <c r="H57" s="15" t="str">
-        <f>G55 &amp; "." &amp; H55 &amp; "-" &amp; H56</f>
+      <c r="H62" s="15" t="str">
+        <f>G60 &amp; "." &amp; H60 &amp; "-" &amp; H61</f>
         <v>v10.0.1-Classic_Reimagined_10</v>
       </c>
-      <c r="I57" s="16"/>
-      <c r="J57" s="14"/>
-    </row>
-    <row r="58" spans="7:10" x14ac:dyDescent="0.3">
-      <c r="G58" s="10" t="s">
-        <v>15</v>
-      </c>
-      <c r="H58" s="15" t="str">
-        <f>H57 &amp; "-build-" &amp; I55</f>
-        <v>v10.0.1-Classic_Reimagined_10-build-6309-rt6</v>
-      </c>
-      <c r="I58" s="16"/>
-    </row>
-    <row r="59" spans="7:10" x14ac:dyDescent="0.3">
-      <c r="G59" s="25" t="s">
-        <v>30</v>
-      </c>
-      <c r="H59" s="25"/>
-      <c r="I59" s="25"/>
-      <c r="J59" s="25"/>
-    </row>
-    <row r="60" spans="7:10" x14ac:dyDescent="0.3">
-      <c r="G60" s="7" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="61" spans="7:10" x14ac:dyDescent="0.3">
-      <c r="G61" s="8" t="s">
-        <v>17</v>
-      </c>
-      <c r="H61" s="8" t="s">
-        <v>6</v>
-      </c>
-      <c r="I61" s="8" t="s">
-        <v>3</v>
-      </c>
-      <c r="J61" s="8" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="62" spans="7:10" x14ac:dyDescent="0.3">
-      <c r="G62" s="9" t="s">
-        <v>32</v>
-      </c>
-      <c r="H62" s="9">
-        <v>32</v>
-      </c>
-      <c r="I62" s="9" t="str">
-        <f>I55</f>
-        <v>6309-rt6</v>
-      </c>
-      <c r="J62" s="9" t="s">
-        <v>33</v>
-      </c>
+      <c r="I62" s="16"/>
+      <c r="J62" s="14"/>
     </row>
     <row r="63" spans="7:10" x14ac:dyDescent="0.3">
       <c r="G63" s="10" t="s">
+        <v>15</v>
+      </c>
+      <c r="H63" s="15" t="str">
+        <f>H62 &amp; "-build-" &amp; I60</f>
+        <v>v10.0.1-Classic_Reimagined_10-build-6410-rt6</v>
+      </c>
+      <c r="I63" s="16"/>
+    </row>
+    <row r="64" spans="7:10" x14ac:dyDescent="0.3">
+      <c r="G64" s="25" t="s">
+        <v>30</v>
+      </c>
+      <c r="H64" s="25"/>
+      <c r="I64" s="25"/>
+      <c r="J64" s="25"/>
+    </row>
+    <row r="65" spans="7:10" x14ac:dyDescent="0.3">
+      <c r="G65" s="7" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="66" spans="7:10" x14ac:dyDescent="0.3">
+      <c r="G66" s="8" t="s">
+        <v>17</v>
+      </c>
+      <c r="H66" s="8" t="s">
+        <v>6</v>
+      </c>
+      <c r="I66" s="8" t="s">
+        <v>3</v>
+      </c>
+      <c r="J66" s="8" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="67" spans="7:10" x14ac:dyDescent="0.3">
+      <c r="G67" s="9" t="s">
+        <v>32</v>
+      </c>
+      <c r="H67" s="9">
+        <v>32</v>
+      </c>
+      <c r="I67" s="9" t="str">
+        <f>I60</f>
+        <v>6410-rt6</v>
+      </c>
+      <c r="J67" s="9" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="68" spans="7:10" x14ac:dyDescent="0.3">
+      <c r="G68" s="10" t="s">
         <v>13</v>
       </c>
-      <c r="H63" s="15" t="s">
+      <c r="H68" s="15" t="s">
         <v>34</v>
       </c>
-      <c r="I63" s="16"/>
-      <c r="J63" s="14"/>
-    </row>
-    <row r="64" spans="7:10" x14ac:dyDescent="0.3">
-      <c r="G64" s="10" t="s">
-        <v>14</v>
-      </c>
-      <c r="H64" s="15" t="str">
-        <f>G62 &amp; "." &amp; H62 &amp; "-" &amp; H63</f>
-        <v>v8.10.32-Classic_Reimagined_8</v>
-      </c>
-      <c r="I64" s="16"/>
-      <c r="J64" s="14"/>
-    </row>
-    <row r="65" spans="7:10" x14ac:dyDescent="0.3">
-      <c r="G65" s="10" t="s">
-        <v>15</v>
-      </c>
-      <c r="H65" s="15" t="str">
-        <f>H64 &amp; "-build-" &amp; I62</f>
-        <v>v8.10.32-Classic_Reimagined_8-build-6309-rt6</v>
-      </c>
-      <c r="I65" s="16"/>
-    </row>
-    <row r="66" spans="7:10" x14ac:dyDescent="0.3">
-      <c r="G66" s="7" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="67" spans="7:10" x14ac:dyDescent="0.3">
-      <c r="G67" s="8" t="s">
-        <v>17</v>
-      </c>
-      <c r="H67" s="8" t="s">
-        <v>6</v>
-      </c>
-      <c r="I67" s="8" t="s">
-        <v>3</v>
-      </c>
-      <c r="J67" s="8" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="68" spans="7:10" x14ac:dyDescent="0.3">
-      <c r="G68" s="9" t="s">
-        <v>32</v>
-      </c>
-      <c r="H68" s="9">
-        <v>31</v>
-      </c>
-      <c r="I68" s="9" t="str">
-        <f>I62</f>
-        <v>6309-rt6</v>
-      </c>
-      <c r="J68" s="9" t="s">
-        <v>35</v>
-      </c>
+      <c r="I68" s="16"/>
+      <c r="J68" s="14"/>
     </row>
     <row r="69" spans="7:10" x14ac:dyDescent="0.3">
       <c r="G69" s="10" t="s">
-        <v>13</v>
-      </c>
-      <c r="H69" s="15" t="s">
-        <v>34</v>
+        <v>14</v>
+      </c>
+      <c r="H69" s="15" t="str">
+        <f>G67 &amp; "." &amp; H67 &amp; "-" &amp; H68</f>
+        <v>v8.10.32-Classic_Reimagined_8</v>
       </c>
       <c r="I69" s="16"/>
       <c r="J69" s="14"/>
     </row>
     <row r="70" spans="7:10" x14ac:dyDescent="0.3">
       <c r="G70" s="10" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="H70" s="15" t="str">
-        <f>G68 &amp; "." &amp; H68 &amp; "-" &amp; H69</f>
-        <v>v8.10.31-Classic_Reimagined_8</v>
+        <f>H69 &amp; "-build-" &amp; I67</f>
+        <v>v8.10.32-Classic_Reimagined_8-build-6410-rt6</v>
       </c>
       <c r="I70" s="16"/>
-      <c r="J70" s="14"/>
     </row>
     <row r="71" spans="7:10" x14ac:dyDescent="0.3">
-      <c r="G71" s="10" t="s">
-        <v>15</v>
-      </c>
-      <c r="H71" s="15" t="str">
-        <f>H70 &amp; "-build-" &amp; I68</f>
-        <v>v8.10.31-Classic_Reimagined_8-build-6309-rt6</v>
-      </c>
-      <c r="I71" s="16"/>
+      <c r="G71" s="7" t="s">
+        <v>31</v>
+      </c>
     </row>
     <row r="72" spans="7:10" x14ac:dyDescent="0.3">
-      <c r="G72" s="26" t="s">
-        <v>36</v>
-      </c>
-      <c r="H72" s="26"/>
-      <c r="I72" s="26"/>
-      <c r="J72" s="26"/>
+      <c r="G72" s="8" t="s">
+        <v>17</v>
+      </c>
+      <c r="H72" s="8" t="s">
+        <v>6</v>
+      </c>
+      <c r="I72" s="8" t="s">
+        <v>3</v>
+      </c>
+      <c r="J72" s="8" t="s">
+        <v>4</v>
+      </c>
     </row>
     <row r="73" spans="7:10" x14ac:dyDescent="0.3">
-      <c r="G73" s="8" t="s">
-        <v>17</v>
-      </c>
-      <c r="H73" s="8" t="s">
-        <v>6</v>
-      </c>
-      <c r="I73" s="8" t="s">
-        <v>3</v>
-      </c>
-      <c r="J73" s="8" t="s">
-        <v>4</v>
+      <c r="G73" s="9" t="s">
+        <v>32</v>
+      </c>
+      <c r="H73" s="9">
+        <v>31</v>
+      </c>
+      <c r="I73" s="9" t="str">
+        <f>I67</f>
+        <v>6410-rt6</v>
+      </c>
+      <c r="J73" s="9" t="s">
+        <v>35</v>
       </c>
     </row>
     <row r="74" spans="7:10" x14ac:dyDescent="0.3">
-      <c r="G74" s="9" t="s">
-        <v>37</v>
-      </c>
-      <c r="H74" s="9">
-        <v>3</v>
-      </c>
-      <c r="I74" s="9" t="str">
-        <f>I68</f>
-        <v>6309-rt6</v>
-      </c>
-      <c r="J74" s="9" t="s">
-        <v>38</v>
-      </c>
+      <c r="G74" s="10" t="s">
+        <v>13</v>
+      </c>
+      <c r="H74" s="15" t="s">
+        <v>34</v>
+      </c>
+      <c r="I74" s="16"/>
+      <c r="J74" s="14"/>
     </row>
     <row r="75" spans="7:10" x14ac:dyDescent="0.3">
       <c r="G75" s="10" t="s">
-        <v>13</v>
-      </c>
-      <c r="H75" s="15" t="s">
-        <v>39</v>
+        <v>14</v>
+      </c>
+      <c r="H75" s="15" t="str">
+        <f>G73 &amp; "." &amp; H73 &amp; "-" &amp; H74</f>
+        <v>v8.10.31-Classic_Reimagined_8</v>
       </c>
       <c r="I75" s="16"/>
       <c r="J75" s="14"/>
     </row>
     <row r="76" spans="7:10" x14ac:dyDescent="0.3">
       <c r="G76" s="10" t="s">
+        <v>15</v>
+      </c>
+      <c r="H76" s="15" t="str">
+        <f>H75 &amp; "-build-" &amp; I73</f>
+        <v>v8.10.31-Classic_Reimagined_8-build-6410-rt6</v>
+      </c>
+      <c r="I76" s="16"/>
+    </row>
+    <row r="77" spans="7:10" x14ac:dyDescent="0.3">
+      <c r="G77" s="26" t="s">
+        <v>36</v>
+      </c>
+      <c r="H77" s="26"/>
+      <c r="I77" s="26"/>
+      <c r="J77" s="26"/>
+    </row>
+    <row r="78" spans="7:10" x14ac:dyDescent="0.3">
+      <c r="G78" s="8" t="s">
+        <v>17</v>
+      </c>
+      <c r="H78" s="8" t="s">
+        <v>6</v>
+      </c>
+      <c r="I78" s="8" t="s">
+        <v>3</v>
+      </c>
+      <c r="J78" s="8" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="79" spans="7:10" x14ac:dyDescent="0.3">
+      <c r="G79" s="9" t="s">
+        <v>37</v>
+      </c>
+      <c r="H79" s="9">
+        <v>3</v>
+      </c>
+      <c r="I79" s="9" t="str">
+        <f>I73</f>
+        <v>6410-rt6</v>
+      </c>
+      <c r="J79" s="9" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="80" spans="7:10" x14ac:dyDescent="0.3">
+      <c r="G80" s="10" t="s">
+        <v>13</v>
+      </c>
+      <c r="H80" s="15" t="s">
+        <v>39</v>
+      </c>
+      <c r="I80" s="16"/>
+      <c r="J80" s="14"/>
+    </row>
+    <row r="81" spans="7:10" x14ac:dyDescent="0.3">
+      <c r="G81" s="10" t="s">
         <v>14</v>
       </c>
-      <c r="H76" s="15" t="str">
-        <f>G74 &amp; "." &amp; H74 &amp; "-" &amp; H75</f>
+      <c r="H81" s="15" t="str">
+        <f>G79 &amp; "." &amp; H79 &amp; "-" &amp; H80</f>
         <v>v7.11.3-Better_Default_7</v>
       </c>
-      <c r="I76" s="16"/>
-      <c r="J76" s="14"/>
-    </row>
-    <row r="77" spans="7:10" x14ac:dyDescent="0.3">
-      <c r="G77" s="10" t="s">
+      <c r="I81" s="16"/>
+      <c r="J81" s="14"/>
+    </row>
+    <row r="82" spans="7:10" x14ac:dyDescent="0.3">
+      <c r="G82" s="10" t="s">
         <v>15</v>
       </c>
-      <c r="H77" s="15" t="str">
-        <f>H76 &amp; "-build-" &amp; I74</f>
-        <v>v7.11.3-Better_Default_7-build-6309-rt6</v>
-      </c>
-      <c r="I77" s="16"/>
+      <c r="H82" s="15" t="str">
+        <f>H81 &amp; "-build-" &amp; I79</f>
+        <v>v7.11.3-Better_Default_7-build-6410-rt6</v>
+      </c>
+      <c r="I82" s="16"/>
     </row>
   </sheetData>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A10:A20">
     <sortCondition ref="A20"/>
   </sortState>
   <mergeCells count="9">
+    <mergeCell ref="G18:K18"/>
+    <mergeCell ref="G64:J64"/>
+    <mergeCell ref="G77:J77"/>
     <mergeCell ref="G1:K1"/>
-    <mergeCell ref="G13:K13"/>
-    <mergeCell ref="G59:J59"/>
-    <mergeCell ref="G72:J72"/>
     <mergeCell ref="A1:E1"/>
     <mergeCell ref="C9:E9"/>
     <mergeCell ref="C10:E10"/>
@@ -2233,11 +2309,6 @@
     </row>
   </sheetData>
   <mergeCells count="17">
-    <mergeCell ref="B41:C41"/>
-    <mergeCell ref="B36:C36"/>
-    <mergeCell ref="B35:C35"/>
-    <mergeCell ref="B31:C31"/>
-    <mergeCell ref="B30:C30"/>
     <mergeCell ref="B10:C10"/>
     <mergeCell ref="B6:C6"/>
     <mergeCell ref="B5:C5"/>
@@ -2250,6 +2321,11 @@
     <mergeCell ref="B16:C16"/>
     <mergeCell ref="B15:C15"/>
     <mergeCell ref="B11:C11"/>
+    <mergeCell ref="B41:C41"/>
+    <mergeCell ref="B36:C36"/>
+    <mergeCell ref="B35:C35"/>
+    <mergeCell ref="B31:C31"/>
+    <mergeCell ref="B30:C30"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait"/>

</xml_diff>

<commit_message>
Added frostbite spawn egg item
</commit_message>
<xml_diff>
--- a/version_guide.xlsx
+++ b/version_guide.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\PrismLauncher\instances\NeoBeta Remastered\minecraft\resourcepacks\Classic-Reimagined\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3651B3C6-EED2-4052-AD8F-02A711BE96CF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D609BB8A-EC46-454E-B569-C700CD9635BB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="521" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="243" uniqueCount="79">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="245" uniqueCount="81">
   <si>
     <t>Current version in development</t>
   </si>
@@ -271,6 +271,12 @@
   </si>
   <si>
     <t>Added 26.4 shader compatibility</t>
+  </si>
+  <si>
+    <t>Compressed textures</t>
+  </si>
+  <si>
+    <t>Added frostbite spawn egg item</t>
   </si>
 </sst>
 </file>
@@ -510,13 +516,13 @@
     <xf numFmtId="1" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -779,13 +785,13 @@
       <c r="C1" s="28"/>
       <c r="D1" s="28"/>
       <c r="E1" s="29"/>
-      <c r="G1" s="24" t="s">
+      <c r="G1" s="26" t="s">
         <v>66</v>
       </c>
-      <c r="H1" s="24"/>
-      <c r="I1" s="24"/>
-      <c r="J1" s="24"/>
-      <c r="K1" s="24"/>
+      <c r="H1" s="26"/>
+      <c r="I1" s="26"/>
+      <c r="J1" s="26"/>
+      <c r="K1" s="26"/>
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A2" s="21" t="s">
@@ -1102,13 +1108,13 @@
       <c r="A18" s="6" t="s">
         <v>77</v>
       </c>
-      <c r="G18" s="25" t="s">
+      <c r="G18" s="24" t="s">
         <v>1</v>
       </c>
-      <c r="H18" s="25"/>
-      <c r="I18" s="25"/>
-      <c r="J18" s="25"/>
-      <c r="K18" s="25"/>
+      <c r="H18" s="24"/>
+      <c r="I18" s="24"/>
+      <c r="J18" s="24"/>
+      <c r="K18" s="24"/>
     </row>
     <row r="19" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A19" s="6" t="s">
@@ -1119,6 +1125,9 @@
       </c>
     </row>
     <row r="20" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A20" s="6" t="s">
+        <v>79</v>
+      </c>
       <c r="G20" s="8" t="s">
         <v>2</v>
       </c>
@@ -1136,6 +1145,9 @@
       </c>
     </row>
     <row r="21" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A21" s="6" t="s">
+        <v>80</v>
+      </c>
       <c r="G21" s="9" t="s">
         <v>11</v>
       </c>
@@ -1634,12 +1646,12 @@
       <c r="I63" s="16"/>
     </row>
     <row r="64" spans="7:10" x14ac:dyDescent="0.3">
-      <c r="G64" s="25" t="s">
+      <c r="G64" s="24" t="s">
         <v>30</v>
       </c>
-      <c r="H64" s="25"/>
-      <c r="I64" s="25"/>
-      <c r="J64" s="25"/>
+      <c r="H64" s="24"/>
+      <c r="I64" s="24"/>
+      <c r="J64" s="24"/>
     </row>
     <row r="65" spans="7:10" x14ac:dyDescent="0.3">
       <c r="G65" s="7" t="s">
@@ -1772,12 +1784,12 @@
       <c r="I76" s="16"/>
     </row>
     <row r="77" spans="7:10" x14ac:dyDescent="0.3">
-      <c r="G77" s="26" t="s">
+      <c r="G77" s="25" t="s">
         <v>36</v>
       </c>
-      <c r="H77" s="26"/>
-      <c r="I77" s="26"/>
-      <c r="J77" s="26"/>
+      <c r="H77" s="25"/>
+      <c r="I77" s="25"/>
+      <c r="J77" s="25"/>
     </row>
     <row r="78" spans="7:10" x14ac:dyDescent="0.3">
       <c r="G78" s="8" t="s">

</xml_diff>

<commit_message>
Added ice ball texture
</commit_message>
<xml_diff>
--- a/version_guide.xlsx
+++ b/version_guide.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\PrismLauncher\instances\NeoBeta Remastered\minecraft\resourcepacks\Classic-Reimagined\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C0AD6806-513F-4247-8943-B48E46DECFEC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5E79D1D6-FAAF-4459-A2A5-3143B36A1FB5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="521" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="246" uniqueCount="82">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="248" uniqueCount="84">
   <si>
     <t>Current version in development</t>
   </si>
@@ -280,6 +280,12 @@
   </si>
   <si>
     <t>Fixed 26.3 shader crash</t>
+  </si>
+  <si>
+    <t>Added brittle ice textures</t>
+  </si>
+  <si>
+    <t>Added iceball texture</t>
   </si>
 </sst>
 </file>
@@ -975,7 +981,7 @@
     </row>
     <row r="10" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A10" s="6" t="s">
-        <v>68</v>
+        <v>78</v>
       </c>
       <c r="C10" s="33" t="s">
         <v>12</v>
@@ -995,7 +1001,7 @@
     </row>
     <row r="11" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A11" s="6" t="s">
-        <v>69</v>
+        <v>82</v>
       </c>
       <c r="G11" s="10" t="s">
         <v>14</v>
@@ -1010,7 +1016,7 @@
     </row>
     <row r="12" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A12" s="6" t="s">
-        <v>70</v>
+        <v>74</v>
       </c>
       <c r="G12" s="10" t="s">
         <v>15</v>
@@ -1024,7 +1030,7 @@
     </row>
     <row r="13" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A13" s="6" t="s">
-        <v>72</v>
+        <v>80</v>
       </c>
       <c r="G13" s="8" t="s">
         <v>2</v>
@@ -1044,7 +1050,7 @@
     </row>
     <row r="14" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A14" s="6" t="s">
-        <v>73</v>
+        <v>83</v>
       </c>
       <c r="G14" s="9" t="s">
         <v>11</v>
@@ -1065,7 +1071,7 @@
     </row>
     <row r="15" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A15" s="6" t="s">
-        <v>74</v>
+        <v>68</v>
       </c>
       <c r="G15" s="10" t="s">
         <v>13</v>
@@ -1080,7 +1086,7 @@
     </row>
     <row r="16" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A16" s="6" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="G16" s="10" t="s">
         <v>14</v>
@@ -1095,7 +1101,7 @@
     </row>
     <row r="17" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A17" s="6" t="s">
-        <v>76</v>
+        <v>79</v>
       </c>
       <c r="G17" s="10" t="s">
         <v>15</v>
@@ -1109,7 +1115,7 @@
     </row>
     <row r="18" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A18" s="6" t="s">
-        <v>77</v>
+        <v>81</v>
       </c>
       <c r="G18" s="24" t="s">
         <v>1</v>
@@ -1121,7 +1127,7 @@
     </row>
     <row r="19" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A19" s="6" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="G19" s="7" t="s">
         <v>5</v>
@@ -1129,7 +1135,7 @@
     </row>
     <row r="20" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A20" s="6" t="s">
-        <v>79</v>
+        <v>75</v>
       </c>
       <c r="G20" s="8" t="s">
         <v>2</v>
@@ -1149,7 +1155,7 @@
     </row>
     <row r="21" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A21" s="6" t="s">
-        <v>80</v>
+        <v>70</v>
       </c>
       <c r="G21" s="9" t="s">
         <v>11</v>
@@ -1170,7 +1176,7 @@
     </row>
     <row r="22" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A22" s="6" t="s">
-        <v>81</v>
+        <v>73</v>
       </c>
       <c r="G22" s="10" t="s">
         <v>13</v>
@@ -1184,6 +1190,9 @@
       <c r="K22" s="14"/>
     </row>
     <row r="23" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A23" s="6" t="s">
+        <v>72</v>
+      </c>
       <c r="G23" s="10" t="s">
         <v>14</v>
       </c>
@@ -1196,6 +1205,9 @@
       <c r="K23" s="14"/>
     </row>
     <row r="24" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A24" s="6" t="s">
+        <v>69</v>
+      </c>
       <c r="G24" s="10" t="s">
         <v>15</v>
       </c>
@@ -1858,8 +1870,8 @@
       <c r="I82" s="16"/>
     </row>
   </sheetData>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A10:A20">
-    <sortCondition ref="A20"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A10:A24">
+    <sortCondition ref="A24"/>
   </sortState>
   <mergeCells count="9">
     <mergeCell ref="G18:K18"/>

</xml_diff>

<commit_message>
added packed ice bricks and chiseled packed ice textures
</commit_message>
<xml_diff>
--- a/version_guide.xlsx
+++ b/version_guide.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\PrismLauncher\instances\NeoBeta Remastered\minecraft\resourcepacks\Classic-Reimagined\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5E79D1D6-FAAF-4459-A2A5-3143B36A1FB5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B3CE4ECE-AE00-43AE-8CED-C91376963F18}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="521" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="248" uniqueCount="84">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="234" uniqueCount="70">
   <si>
     <t>Current version in development</t>
   </si>
@@ -240,59 +240,17 @@
     <t>Release year</t>
   </si>
   <si>
-    <t>Added map textures</t>
-  </si>
-  <si>
-    <t>Updated fog shaders</t>
-  </si>
-  <si>
-    <t>Fixed texture sampling (26.3+ only)</t>
-  </si>
-  <si>
     <t>_11_Beta</t>
   </si>
   <si>
-    <t>Renamed resource pack</t>
-  </si>
-  <si>
-    <t>Removed nether fog</t>
-  </si>
-  <si>
-    <t>Added exponential fog</t>
-  </si>
-  <si>
-    <t>Fixed hyper-realistic fog</t>
-  </si>
-  <si>
-    <t>Changed underwater fog color</t>
-  </si>
-  <si>
-    <t>Fixed baby rabbit model</t>
-  </si>
-  <si>
-    <t>Added 26.4 shader compatibility</t>
-  </si>
-  <si>
-    <t>Compressed textures</t>
-  </si>
-  <si>
-    <t>Added frostbite spawn egg item</t>
-  </si>
-  <si>
-    <t>Fixed 26.3 shader crash</t>
-  </si>
-  <si>
-    <t>Added brittle ice textures</t>
-  </si>
-  <si>
-    <t>Added iceball texture</t>
+    <t>Added packed ice bricks and chiseled packed ice textures</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="9" x14ac:knownFonts="1">
+  <fonts count="10" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -343,6 +301,12 @@
     <font>
       <sz val="11"/>
       <color theme="0"/>
+      <name val="Segoe UI"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color theme="1"/>
       <name val="Segoe UI"/>
       <family val="2"/>
     </font>
@@ -480,7 +444,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="45">
+  <cellXfs count="46">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
@@ -588,6 +552,7 @@
     <xf numFmtId="0" fontId="1" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -810,7 +775,7 @@
         <v>6</v>
       </c>
       <c r="G2" s="7" t="s">
-        <v>71</v>
+        <v>68</v>
       </c>
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.3">
@@ -841,7 +806,7 @@
         <v>63</v>
       </c>
       <c r="B4" s="22">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="G4" s="9" t="s">
         <v>11</v>
@@ -854,10 +819,10 @@
       </c>
       <c r="J4" s="9" t="str">
         <f>D8</f>
-        <v>6410-rt6</v>
+        <v>6411-rt6</v>
       </c>
       <c r="K4" s="9">
-        <v>26.3</v>
+        <v>26.4</v>
       </c>
     </row>
     <row r="5" spans="1:11" x14ac:dyDescent="0.3">
@@ -884,7 +849,7 @@
       </c>
       <c r="B6" s="23">
         <f>(B2*1000)+(B3*100)+B4+((B5-2026)*1000)</f>
-        <v>6410</v>
+        <v>6411</v>
       </c>
       <c r="G6" s="10" t="s">
         <v>14</v>
@@ -914,7 +879,7 @@
       </c>
       <c r="H7" s="11" t="str">
         <f>H6 &amp; "-build-" &amp; J4</f>
-        <v>v10.0.11_4-DogePack_Classic_11_Beta-build-6410-rt6</v>
+        <v>v10.0.11_4-DogePack_Classic_11_Beta-build-6411-rt6</v>
       </c>
       <c r="I7" s="12"/>
       <c r="J7" s="13"/>
@@ -922,17 +887,17 @@
     <row r="8" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A8" s="39" t="str">
         <f>G4 &amp; "." &amp; H4 &amp; "_" &amp; I4 &amp; "-build-" &amp; D8</f>
-        <v>v10.0.11_4-build-6410-rt6</v>
+        <v>v10.0.11_4-build-6411-rt6</v>
       </c>
       <c r="B8" s="40"/>
       <c r="C8" s="41"/>
       <c r="D8" s="9" t="str">
         <f>B6&amp;"-rt"&amp;B2</f>
-        <v>6410-rt6</v>
+        <v>6411-rt6</v>
       </c>
       <c r="E8" s="18">
-        <f>K14</f>
-        <v>26.3</v>
+        <f>K4</f>
+        <v>26.4</v>
       </c>
       <c r="G8" s="8" t="s">
         <v>2</v>
@@ -973,15 +938,15 @@
       </c>
       <c r="J9" s="9" t="str">
         <f>J4</f>
-        <v>6410-rt6</v>
+        <v>6411-rt6</v>
       </c>
       <c r="K9" s="9">
         <v>26.3</v>
       </c>
     </row>
-    <row r="10" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A10" s="6" t="s">
-        <v>78</v>
+    <row r="10" spans="1:11" ht="17.25" x14ac:dyDescent="0.3">
+      <c r="A10" s="45" t="s">
+        <v>69</v>
       </c>
       <c r="C10" s="33" t="s">
         <v>12</v>
@@ -1000,9 +965,6 @@
       <c r="K10" s="14"/>
     </row>
     <row r="11" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A11" s="6" t="s">
-        <v>82</v>
-      </c>
       <c r="G11" s="10" t="s">
         <v>14</v>
       </c>
@@ -1015,23 +977,17 @@
       <c r="K11" s="14"/>
     </row>
     <row r="12" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A12" s="6" t="s">
-        <v>74</v>
-      </c>
       <c r="G12" s="10" t="s">
         <v>15</v>
       </c>
       <c r="H12" s="11" t="str">
         <f>H11 &amp; "-build-" &amp; J9</f>
-        <v>v10.0.11_3-DogePack_ClassicResource Pack Build-build-6410-rt6</v>
+        <v>v10.0.11_3-DogePack_ClassicResource Pack Build-build-6411-rt6</v>
       </c>
       <c r="I12" s="12"/>
       <c r="J12" s="13"/>
     </row>
     <row r="13" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A13" s="6" t="s">
-        <v>80</v>
-      </c>
       <c r="G13" s="8" t="s">
         <v>2</v>
       </c>
@@ -1049,9 +1005,6 @@
       </c>
     </row>
     <row r="14" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A14" s="6" t="s">
-        <v>83</v>
-      </c>
       <c r="G14" s="9" t="s">
         <v>11</v>
       </c>
@@ -1063,16 +1016,13 @@
       </c>
       <c r="J14" s="9" t="str">
         <f>J9</f>
-        <v>6410-rt6</v>
+        <v>6411-rt6</v>
       </c>
       <c r="K14" s="9">
-        <v>26.3</v>
+        <v>26.2</v>
       </c>
     </row>
     <row r="15" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A15" s="6" t="s">
-        <v>68</v>
-      </c>
       <c r="G15" s="10" t="s">
         <v>13</v>
       </c>
@@ -1085,9 +1035,6 @@
       <c r="K15" s="14"/>
     </row>
     <row r="16" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A16" s="6" t="s">
-        <v>76</v>
-      </c>
       <c r="G16" s="10" t="s">
         <v>14</v>
       </c>
@@ -1099,24 +1046,18 @@
       <c r="J16" s="13"/>
       <c r="K16" s="14"/>
     </row>
-    <row r="17" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A17" s="6" t="s">
-        <v>79</v>
-      </c>
+    <row r="17" spans="7:11" x14ac:dyDescent="0.3">
       <c r="G17" s="10" t="s">
         <v>15</v>
       </c>
       <c r="H17" s="11" t="str">
         <f>H16 &amp; "-build-" &amp; J14</f>
-        <v>v10.0.11_2-DogePack_Classic_11_Beta-build-6410-rt6</v>
+        <v>v10.0.11_2-DogePack_Classic_11_Beta-build-6411-rt6</v>
       </c>
       <c r="I17" s="12"/>
       <c r="J17" s="13"/>
     </row>
-    <row r="18" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A18" s="6" t="s">
-        <v>81</v>
-      </c>
+    <row r="18" spans="7:11" x14ac:dyDescent="0.3">
       <c r="G18" s="24" t="s">
         <v>1</v>
       </c>
@@ -1125,18 +1066,12 @@
       <c r="J18" s="24"/>
       <c r="K18" s="24"/>
     </row>
-    <row r="19" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A19" s="6" t="s">
-        <v>77</v>
-      </c>
+    <row r="19" spans="7:11" x14ac:dyDescent="0.3">
       <c r="G19" s="7" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="20" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A20" s="6" t="s">
-        <v>75</v>
-      </c>
+    <row r="20" spans="7:11" x14ac:dyDescent="0.3">
       <c r="G20" s="8" t="s">
         <v>2</v>
       </c>
@@ -1153,10 +1088,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="21" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A21" s="6" t="s">
-        <v>70</v>
-      </c>
+    <row r="21" spans="7:11" x14ac:dyDescent="0.3">
       <c r="G21" s="9" t="s">
         <v>11</v>
       </c>
@@ -1168,16 +1100,13 @@
       </c>
       <c r="J21" s="9" t="str">
         <f>J14</f>
-        <v>6410-rt6</v>
+        <v>6411-rt6</v>
       </c>
       <c r="K21" s="9">
         <v>26.1</v>
       </c>
     </row>
-    <row r="22" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A22" s="6" t="s">
-        <v>73</v>
-      </c>
+    <row r="22" spans="7:11" x14ac:dyDescent="0.3">
       <c r="G22" s="10" t="s">
         <v>13</v>
       </c>
@@ -1189,10 +1118,7 @@
       <c r="J22" s="13"/>
       <c r="K22" s="14"/>
     </row>
-    <row r="23" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A23" s="6" t="s">
-        <v>72</v>
-      </c>
+    <row r="23" spans="7:11" x14ac:dyDescent="0.3">
       <c r="G23" s="10" t="s">
         <v>14</v>
       </c>
@@ -1204,26 +1130,23 @@
       <c r="J23" s="13"/>
       <c r="K23" s="14"/>
     </row>
-    <row r="24" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A24" s="6" t="s">
-        <v>69</v>
-      </c>
+    <row r="24" spans="7:11" x14ac:dyDescent="0.3">
       <c r="G24" s="10" t="s">
         <v>15</v>
       </c>
       <c r="H24" s="11" t="str">
         <f>H23 &amp; "-build-" &amp; J21</f>
-        <v>v10.0.11_1-Classic_Reimagined_10_SE_2.1-build-6410-rt6</v>
+        <v>v10.0.11_1-Classic_Reimagined_10_SE_2.1-build-6411-rt6</v>
       </c>
       <c r="I24" s="12"/>
       <c r="J24" s="13"/>
     </row>
-    <row r="25" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="25" spans="7:11" x14ac:dyDescent="0.3">
       <c r="G25" s="7" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="26" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="26" spans="7:11" x14ac:dyDescent="0.3">
       <c r="G26" s="8" t="s">
         <v>17</v>
       </c>
@@ -1237,7 +1160,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="27" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="27" spans="7:11" x14ac:dyDescent="0.3">
       <c r="G27" s="9" t="s">
         <v>11</v>
       </c>
@@ -1246,13 +1169,13 @@
       </c>
       <c r="I27" s="9" t="str">
         <f>J21</f>
-        <v>6410-rt6</v>
+        <v>6411-rt6</v>
       </c>
       <c r="J27" s="9" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="28" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="28" spans="7:11" x14ac:dyDescent="0.3">
       <c r="G28" s="10" t="s">
         <v>13</v>
       </c>
@@ -1263,7 +1186,7 @@
       <c r="I28" s="16"/>
       <c r="J28" s="14"/>
     </row>
-    <row r="29" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="29" spans="7:11" x14ac:dyDescent="0.3">
       <c r="G29" s="10" t="s">
         <v>14</v>
       </c>
@@ -1274,17 +1197,17 @@
       <c r="I29" s="16"/>
       <c r="J29" s="14"/>
     </row>
-    <row r="30" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="30" spans="7:11" x14ac:dyDescent="0.3">
       <c r="G30" s="10" t="s">
         <v>15</v>
       </c>
       <c r="H30" s="15" t="str">
         <f>H29 &amp; "-build-" &amp; I27</f>
-        <v>v10.0.10-Classic_Reimagined_10_SE_2-build-6410-rt6</v>
+        <v>v10.0.10-Classic_Reimagined_10_SE_2-build-6411-rt6</v>
       </c>
       <c r="I30" s="16"/>
     </row>
-    <row r="31" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="31" spans="7:11" x14ac:dyDescent="0.3">
       <c r="G31" s="8" t="s">
         <v>17</v>
       </c>
@@ -1298,7 +1221,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="32" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="32" spans="7:11" x14ac:dyDescent="0.3">
       <c r="G32" s="9" t="s">
         <v>11</v>
       </c>
@@ -1307,7 +1230,7 @@
       </c>
       <c r="I32" s="9" t="str">
         <f>I27</f>
-        <v>6410-rt6</v>
+        <v>6411-rt6</v>
       </c>
       <c r="J32" s="9" t="s">
         <v>19</v>
@@ -1341,7 +1264,7 @@
       </c>
       <c r="H35" s="15" t="str">
         <f>H34 &amp; "-build-" &amp; I32</f>
-        <v>v10.0.9-Classic_Reimagined_10_SE_2-build-6410-rt6</v>
+        <v>v10.0.9-Classic_Reimagined_10_SE_2-build-6411-rt6</v>
       </c>
       <c r="I35" s="16"/>
     </row>
@@ -1368,7 +1291,7 @@
       </c>
       <c r="I37" s="9" t="str">
         <f>I32</f>
-        <v>6410-rt6</v>
+        <v>6411-rt6</v>
       </c>
       <c r="J37" s="9" t="s">
         <v>20</v>
@@ -1402,7 +1325,7 @@
       </c>
       <c r="H40" s="15" t="str">
         <f>H39 &amp; "-build-" &amp; I37</f>
-        <v>v10.0.7-Classic_Reimagined_10_SE_2-build-6410-rt6</v>
+        <v>v10.0.7-Classic_Reimagined_10_SE_2-build-6411-rt6</v>
       </c>
       <c r="I40" s="16"/>
     </row>
@@ -1429,7 +1352,7 @@
       </c>
       <c r="I42" s="9" t="str">
         <f>I37</f>
-        <v>6410-rt6</v>
+        <v>6411-rt6</v>
       </c>
       <c r="J42" s="9" t="s">
         <v>21</v>
@@ -1463,7 +1386,7 @@
       </c>
       <c r="H45" s="15" t="str">
         <f>H44 &amp; "-build-" &amp; I42</f>
-        <v>v10.0.4-Classic_Reimagined_10_SE_2-build-6410-rt6</v>
+        <v>v10.0.4-Classic_Reimagined_10_SE_2-build-6411-rt6</v>
       </c>
       <c r="I45" s="16"/>
     </row>
@@ -1495,7 +1418,7 @@
       </c>
       <c r="I48" s="9" t="str">
         <f>I42</f>
-        <v>6410-rt6</v>
+        <v>6411-rt6</v>
       </c>
       <c r="J48" s="9" t="s">
         <v>23</v>
@@ -1529,7 +1452,7 @@
       </c>
       <c r="H51" s="15" t="str">
         <f>H50 &amp; "-build-" &amp; I48</f>
-        <v>v10.0.3-Classic_Reimagined_10_SE-build-6410-rt6</v>
+        <v>v10.0.3-Classic_Reimagined_10_SE-build-6411-rt6</v>
       </c>
       <c r="I51" s="16"/>
     </row>
@@ -1561,7 +1484,7 @@
       </c>
       <c r="I54" s="9" t="str">
         <f>I48</f>
-        <v>6410-rt6</v>
+        <v>6411-rt6</v>
       </c>
       <c r="J54" s="9" t="s">
         <v>25</v>
@@ -1594,7 +1517,7 @@
       </c>
       <c r="H57" s="15" t="str">
         <f>H56 &amp; "-build-" &amp; I54</f>
-        <v>v10.0.2-Classic_Reimagined_10s-build-6410-rt6</v>
+        <v>v10.0.2-Classic_Reimagined_10s-build-6411-rt6</v>
       </c>
       <c r="I57" s="16"/>
     </row>
@@ -1626,7 +1549,7 @@
       </c>
       <c r="I60" s="9" t="str">
         <f>I54</f>
-        <v>6410-rt6</v>
+        <v>6411-rt6</v>
       </c>
       <c r="J60" s="9" t="s">
         <v>28</v>
@@ -1659,7 +1582,7 @@
       </c>
       <c r="H63" s="15" t="str">
         <f>H62 &amp; "-build-" &amp; I60</f>
-        <v>v10.0.1-Classic_Reimagined_10-build-6410-rt6</v>
+        <v>v10.0.1-Classic_Reimagined_10-build-6411-rt6</v>
       </c>
       <c r="I63" s="16"/>
     </row>
@@ -1699,7 +1622,7 @@
       </c>
       <c r="I67" s="9" t="str">
         <f>I60</f>
-        <v>6410-rt6</v>
+        <v>6411-rt6</v>
       </c>
       <c r="J67" s="9" t="s">
         <v>33</v>
@@ -1732,7 +1655,7 @@
       </c>
       <c r="H70" s="15" t="str">
         <f>H69 &amp; "-build-" &amp; I67</f>
-        <v>v8.10.32-Classic_Reimagined_8-build-6410-rt6</v>
+        <v>v8.10.32-Classic_Reimagined_8-build-6411-rt6</v>
       </c>
       <c r="I70" s="16"/>
     </row>
@@ -1764,7 +1687,7 @@
       </c>
       <c r="I73" s="9" t="str">
         <f>I67</f>
-        <v>6410-rt6</v>
+        <v>6411-rt6</v>
       </c>
       <c r="J73" s="9" t="s">
         <v>35</v>
@@ -1797,7 +1720,7 @@
       </c>
       <c r="H76" s="15" t="str">
         <f>H75 &amp; "-build-" &amp; I73</f>
-        <v>v8.10.31-Classic_Reimagined_8-build-6410-rt6</v>
+        <v>v8.10.31-Classic_Reimagined_8-build-6411-rt6</v>
       </c>
       <c r="I76" s="16"/>
     </row>
@@ -1832,7 +1755,7 @@
       </c>
       <c r="I79" s="9" t="str">
         <f>I73</f>
-        <v>6410-rt6</v>
+        <v>6411-rt6</v>
       </c>
       <c r="J79" s="9" t="s">
         <v>38</v>
@@ -1865,7 +1788,7 @@
       </c>
       <c r="H82" s="15" t="str">
         <f>H81 &amp; "-build-" &amp; I79</f>
-        <v>v7.11.3-Better_Default_7-build-6410-rt6</v>
+        <v>v7.11.3-Better_Default_7-build-6411-rt6</v>
       </c>
       <c r="I82" s="16"/>
     </row>
@@ -2339,11 +2262,6 @@
     </row>
   </sheetData>
   <mergeCells count="17">
-    <mergeCell ref="B41:C41"/>
-    <mergeCell ref="B36:C36"/>
-    <mergeCell ref="B35:C35"/>
-    <mergeCell ref="B31:C31"/>
-    <mergeCell ref="B30:C30"/>
     <mergeCell ref="B10:C10"/>
     <mergeCell ref="B6:C6"/>
     <mergeCell ref="B5:C5"/>
@@ -2356,6 +2274,11 @@
     <mergeCell ref="B16:C16"/>
     <mergeCell ref="B15:C15"/>
     <mergeCell ref="B11:C11"/>
+    <mergeCell ref="B41:C41"/>
+    <mergeCell ref="B36:C36"/>
+    <mergeCell ref="B35:C35"/>
+    <mergeCell ref="B31:C31"/>
+    <mergeCell ref="B30:C30"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait"/>

</xml_diff>

<commit_message>
changed packed ice and blue ice textures
</commit_message>
<xml_diff>
--- a/version_guide.xlsx
+++ b/version_guide.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\PrismLauncher\instances\NeoBeta Remastered\minecraft\resourcepacks\Classic-Reimagined\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B3CE4ECE-AE00-43AE-8CED-C91376963F18}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3869D4A7-61B9-4CA2-88E1-840EB44DF478}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="521" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="234" uniqueCount="70">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="236" uniqueCount="72">
   <si>
     <t>Current version in development</t>
   </si>
@@ -244,13 +244,19 @@
   </si>
   <si>
     <t>Added packed ice bricks and chiseled packed ice textures</t>
+  </si>
+  <si>
+    <t>Changed packed ice and blue ice textures</t>
+  </si>
+  <si>
+    <t>Added brittle ice textures</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="10" x14ac:knownFonts="1">
+  <fonts count="9" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -273,40 +279,34 @@
       <name val="Segoe UI"/>
     </font>
     <font>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Segoe UI"/>
+      <family val="2"/>
+    </font>
+    <font>
       <b/>
-      <sz val="11"/>
+      <sz val="12"/>
       <color theme="0"/>
       <name val="Segoe UI"/>
       <family val="2"/>
     </font>
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
+      <sz val="12"/>
+      <color theme="0"/>
       <name val="Segoe UI"/>
       <family val="2"/>
     </font>
     <font>
-      <sz val="11"/>
+      <sz val="12"/>
       <color indexed="64"/>
       <name val="Segoe UI"/>
       <family val="2"/>
     </font>
     <font>
       <b/>
-      <sz val="11"/>
+      <sz val="12"/>
       <color indexed="65"/>
-      <name val="Segoe UI"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="0"/>
-      <name val="Segoe UI"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <sz val="12"/>
-      <color theme="1"/>
       <name val="Segoe UI"/>
       <family val="2"/>
     </font>
@@ -444,7 +444,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="46">
+  <cellXfs count="45">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
@@ -455,92 +455,92 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="6" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="1" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="8" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="49" fontId="7" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="8" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="1" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="7" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="7" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="7" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="7" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -552,7 +552,6 @@
     <xf numFmtId="0" fontId="1" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -744,7 +743,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:K82"/>
-  <sheetFormatPr defaultColWidth="27.28515625" defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="27.28515625" defaultRowHeight="17.25" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="36.5703125" style="6" customWidth="1"/>
     <col min="2" max="2" width="36.7109375" style="6" customWidth="1"/>
@@ -768,99 +767,99 @@
       <c r="K1" s="26"/>
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A2" s="21" t="s">
+      <c r="A2" s="7" t="s">
         <v>62</v>
       </c>
-      <c r="B2" s="22">
+      <c r="B2" s="8">
         <v>6</v>
       </c>
-      <c r="G2" s="7" t="s">
+      <c r="G2" s="9" t="s">
         <v>68</v>
       </c>
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A3" s="21" t="s">
+      <c r="A3" s="7" t="s">
         <v>64</v>
       </c>
-      <c r="B3" s="22">
-        <v>4</v>
-      </c>
-      <c r="G3" s="8" t="s">
+      <c r="B3" s="8">
+        <v>4</v>
+      </c>
+      <c r="G3" s="10" t="s">
         <v>2</v>
       </c>
-      <c r="H3" s="8" t="s">
+      <c r="H3" s="10" t="s">
         <v>6</v>
       </c>
-      <c r="I3" s="8" t="s">
+      <c r="I3" s="10" t="s">
         <v>7</v>
       </c>
-      <c r="J3" s="8" t="s">
+      <c r="J3" s="10" t="s">
         <v>3</v>
       </c>
-      <c r="K3" s="8" t="s">
+      <c r="K3" s="10" t="s">
         <v>4</v>
       </c>
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A4" s="21" t="s">
+      <c r="A4" s="7" t="s">
         <v>63</v>
       </c>
-      <c r="B4" s="22">
+      <c r="B4" s="8">
         <v>11</v>
       </c>
-      <c r="G4" s="9" t="s">
+      <c r="G4" s="11" t="s">
         <v>11</v>
       </c>
-      <c r="H4" s="9">
+      <c r="H4" s="11">
         <v>11</v>
       </c>
-      <c r="I4" s="9">
-        <v>4</v>
-      </c>
-      <c r="J4" s="9" t="str">
+      <c r="I4" s="11">
+        <v>4</v>
+      </c>
+      <c r="J4" s="11" t="str">
         <f>D8</f>
         <v>6411-rt6</v>
       </c>
-      <c r="K4" s="9">
+      <c r="K4" s="11">
         <v>26.4</v>
       </c>
     </row>
     <row r="5" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A5" s="21" t="s">
+      <c r="A5" s="7" t="s">
         <v>67</v>
       </c>
-      <c r="B5" s="22">
+      <c r="B5" s="8">
         <v>2026</v>
       </c>
-      <c r="G5" s="10" t="s">
+      <c r="G5" s="12" t="s">
         <v>13</v>
       </c>
-      <c r="H5" s="11" t="str">
+      <c r="H5" s="13" t="str">
         <f>"DogePack_Classic" &amp; G2</f>
         <v>DogePack_Classic_11_Beta</v>
       </c>
-      <c r="I5" s="12"/>
-      <c r="J5" s="13"/>
-      <c r="K5" s="14"/>
+      <c r="I5" s="14"/>
+      <c r="J5" s="15"/>
+      <c r="K5" s="16"/>
     </row>
     <row r="6" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A6" s="21" t="s">
+      <c r="A6" s="7" t="s">
         <v>65</v>
       </c>
-      <c r="B6" s="23">
+      <c r="B6" s="17">
         <f>(B2*1000)+(B3*100)+B4+((B5-2026)*1000)</f>
         <v>6411</v>
       </c>
-      <c r="G6" s="10" t="s">
+      <c r="G6" s="12" t="s">
         <v>14</v>
       </c>
-      <c r="H6" s="11" t="str">
+      <c r="H6" s="13" t="str">
         <f>G4 &amp; "." &amp; H4 &amp; "_" &amp; I4 &amp; "-" &amp; H5</f>
         <v>v10.0.11_4-DogePack_Classic_11_Beta</v>
       </c>
-      <c r="I6" s="12"/>
-      <c r="J6" s="13"/>
-      <c r="K6" s="14"/>
+      <c r="I6" s="14"/>
+      <c r="J6" s="15"/>
+      <c r="K6" s="16"/>
     </row>
     <row r="7" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A7" s="36" t="s">
@@ -868,21 +867,21 @@
       </c>
       <c r="B7" s="37"/>
       <c r="C7" s="38"/>
-      <c r="D7" s="8" t="s">
+      <c r="D7" s="10" t="s">
         <v>3</v>
       </c>
-      <c r="E7" s="17" t="s">
-        <v>4</v>
-      </c>
-      <c r="G7" s="10" t="s">
+      <c r="E7" s="18" t="s">
+        <v>4</v>
+      </c>
+      <c r="G7" s="12" t="s">
         <v>15</v>
       </c>
-      <c r="H7" s="11" t="str">
+      <c r="H7" s="13" t="str">
         <f>H6 &amp; "-build-" &amp; J4</f>
         <v>v10.0.11_4-DogePack_Classic_11_Beta-build-6411-rt6</v>
       </c>
-      <c r="I7" s="12"/>
-      <c r="J7" s="13"/>
+      <c r="I7" s="14"/>
+      <c r="J7" s="15"/>
     </row>
     <row r="8" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A8" s="39" t="str">
@@ -891,35 +890,35 @@
       </c>
       <c r="B8" s="40"/>
       <c r="C8" s="41"/>
-      <c r="D8" s="9" t="str">
+      <c r="D8" s="11" t="str">
         <f>B6&amp;"-rt"&amp;B2</f>
         <v>6411-rt6</v>
       </c>
-      <c r="E8" s="18">
+      <c r="E8" s="19">
         <f>K4</f>
         <v>26.4</v>
       </c>
-      <c r="G8" s="8" t="s">
+      <c r="G8" s="10" t="s">
         <v>2</v>
       </c>
-      <c r="H8" s="8" t="s">
+      <c r="H8" s="10" t="s">
         <v>6</v>
       </c>
-      <c r="I8" s="8" t="s">
+      <c r="I8" s="10" t="s">
         <v>7</v>
       </c>
-      <c r="J8" s="8" t="s">
+      <c r="J8" s="10" t="s">
         <v>3</v>
       </c>
-      <c r="K8" s="8" t="s">
+      <c r="K8" s="10" t="s">
         <v>4</v>
       </c>
     </row>
     <row r="9" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A9" s="19" t="s">
+      <c r="A9" s="20" t="s">
         <v>8</v>
       </c>
-      <c r="B9" s="20" t="s">
+      <c r="B9" s="21" t="s">
         <v>9</v>
       </c>
       <c r="C9" s="30" t="s">
@@ -927,25 +926,25 @@
       </c>
       <c r="D9" s="31"/>
       <c r="E9" s="32"/>
-      <c r="G9" s="9" t="s">
+      <c r="G9" s="11" t="s">
         <v>11</v>
       </c>
-      <c r="H9" s="9">
+      <c r="H9" s="11">
         <v>11</v>
       </c>
-      <c r="I9" s="9">
+      <c r="I9" s="11">
         <v>3</v>
       </c>
-      <c r="J9" s="9" t="str">
+      <c r="J9" s="11" t="str">
         <f>J4</f>
         <v>6411-rt6</v>
       </c>
-      <c r="K9" s="9">
+      <c r="K9" s="11">
         <v>26.3</v>
       </c>
     </row>
-    <row r="10" spans="1:11" ht="17.25" x14ac:dyDescent="0.3">
-      <c r="A10" s="45" t="s">
+    <row r="10" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A10" s="6" t="s">
         <v>69</v>
       </c>
       <c r="C10" s="33" t="s">
@@ -953,109 +952,115 @@
       </c>
       <c r="D10" s="34"/>
       <c r="E10" s="35"/>
-      <c r="G10" s="10" t="s">
+      <c r="G10" s="12" t="s">
         <v>13</v>
       </c>
-      <c r="H10" s="11" t="str">
+      <c r="H10" s="13" t="str">
         <f>"DogePack_Classic" &amp; G7</f>
         <v>DogePack_ClassicResource Pack Build</v>
       </c>
-      <c r="I10" s="12"/>
-      <c r="J10" s="13"/>
-      <c r="K10" s="14"/>
+      <c r="I10" s="14"/>
+      <c r="J10" s="15"/>
+      <c r="K10" s="16"/>
     </row>
     <row r="11" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="G11" s="10" t="s">
+      <c r="A11" s="6" t="s">
+        <v>70</v>
+      </c>
+      <c r="G11" s="12" t="s">
         <v>14</v>
       </c>
-      <c r="H11" s="11" t="str">
+      <c r="H11" s="13" t="str">
         <f>G9 &amp; "." &amp; H9 &amp; "_" &amp; I9 &amp; "-" &amp; H10</f>
         <v>v10.0.11_3-DogePack_ClassicResource Pack Build</v>
       </c>
-      <c r="I11" s="12"/>
-      <c r="J11" s="13"/>
-      <c r="K11" s="14"/>
+      <c r="I11" s="14"/>
+      <c r="J11" s="15"/>
+      <c r="K11" s="16"/>
     </row>
     <row r="12" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="G12" s="10" t="s">
+      <c r="A12" s="6" t="s">
+        <v>71</v>
+      </c>
+      <c r="G12" s="12" t="s">
         <v>15</v>
       </c>
-      <c r="H12" s="11" t="str">
+      <c r="H12" s="13" t="str">
         <f>H11 &amp; "-build-" &amp; J9</f>
         <v>v10.0.11_3-DogePack_ClassicResource Pack Build-build-6411-rt6</v>
       </c>
-      <c r="I12" s="12"/>
-      <c r="J12" s="13"/>
+      <c r="I12" s="14"/>
+      <c r="J12" s="15"/>
     </row>
     <row r="13" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="G13" s="8" t="s">
+      <c r="G13" s="10" t="s">
         <v>2</v>
       </c>
-      <c r="H13" s="8" t="s">
+      <c r="H13" s="10" t="s">
         <v>6</v>
       </c>
-      <c r="I13" s="8" t="s">
+      <c r="I13" s="10" t="s">
         <v>7</v>
       </c>
-      <c r="J13" s="8" t="s">
+      <c r="J13" s="10" t="s">
         <v>3</v>
       </c>
-      <c r="K13" s="8" t="s">
+      <c r="K13" s="10" t="s">
         <v>4</v>
       </c>
     </row>
     <row r="14" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="G14" s="9" t="s">
+      <c r="G14" s="11" t="s">
         <v>11</v>
       </c>
-      <c r="H14" s="9">
+      <c r="H14" s="11">
         <v>11</v>
       </c>
-      <c r="I14" s="9">
+      <c r="I14" s="11">
         <v>2</v>
       </c>
-      <c r="J14" s="9" t="str">
+      <c r="J14" s="11" t="str">
         <f>J9</f>
         <v>6411-rt6</v>
       </c>
-      <c r="K14" s="9">
+      <c r="K14" s="11">
         <v>26.2</v>
       </c>
     </row>
     <row r="15" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="G15" s="10" t="s">
+      <c r="G15" s="12" t="s">
         <v>13</v>
       </c>
-      <c r="H15" s="11" t="str">
+      <c r="H15" s="13" t="str">
         <f>H5</f>
         <v>DogePack_Classic_11_Beta</v>
       </c>
-      <c r="I15" s="12"/>
-      <c r="J15" s="13"/>
-      <c r="K15" s="14"/>
+      <c r="I15" s="14"/>
+      <c r="J15" s="15"/>
+      <c r="K15" s="16"/>
     </row>
     <row r="16" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="G16" s="10" t="s">
+      <c r="G16" s="12" t="s">
         <v>14</v>
       </c>
-      <c r="H16" s="11" t="str">
+      <c r="H16" s="13" t="str">
         <f>G14 &amp; "." &amp; H14 &amp; "_" &amp; I14 &amp; "-" &amp; H15</f>
         <v>v10.0.11_2-DogePack_Classic_11_Beta</v>
       </c>
-      <c r="I16" s="12"/>
-      <c r="J16" s="13"/>
-      <c r="K16" s="14"/>
+      <c r="I16" s="14"/>
+      <c r="J16" s="15"/>
+      <c r="K16" s="16"/>
     </row>
     <row r="17" spans="7:11" x14ac:dyDescent="0.3">
-      <c r="G17" s="10" t="s">
+      <c r="G17" s="12" t="s">
         <v>15</v>
       </c>
-      <c r="H17" s="11" t="str">
+      <c r="H17" s="13" t="str">
         <f>H16 &amp; "-build-" &amp; J14</f>
         <v>v10.0.11_2-DogePack_Classic_11_Beta-build-6411-rt6</v>
       </c>
-      <c r="I17" s="12"/>
-      <c r="J17" s="13"/>
+      <c r="I17" s="14"/>
+      <c r="J17" s="15"/>
     </row>
     <row r="18" spans="7:11" x14ac:dyDescent="0.3">
       <c r="G18" s="24" t="s">
@@ -1067,524 +1072,524 @@
       <c r="K18" s="24"/>
     </row>
     <row r="19" spans="7:11" x14ac:dyDescent="0.3">
-      <c r="G19" s="7" t="s">
+      <c r="G19" s="9" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="20" spans="7:11" x14ac:dyDescent="0.3">
-      <c r="G20" s="8" t="s">
+      <c r="G20" s="10" t="s">
         <v>2</v>
       </c>
-      <c r="H20" s="8" t="s">
+      <c r="H20" s="10" t="s">
         <v>6</v>
       </c>
-      <c r="I20" s="8" t="s">
+      <c r="I20" s="10" t="s">
         <v>7</v>
       </c>
-      <c r="J20" s="8" t="s">
+      <c r="J20" s="10" t="s">
         <v>3</v>
       </c>
-      <c r="K20" s="8" t="s">
+      <c r="K20" s="10" t="s">
         <v>4</v>
       </c>
     </row>
     <row r="21" spans="7:11" x14ac:dyDescent="0.3">
-      <c r="G21" s="9" t="s">
+      <c r="G21" s="11" t="s">
         <v>11</v>
       </c>
-      <c r="H21" s="9">
+      <c r="H21" s="11">
         <v>11</v>
       </c>
-      <c r="I21" s="9">
+      <c r="I21" s="11">
         <v>1</v>
       </c>
-      <c r="J21" s="9" t="str">
+      <c r="J21" s="11" t="str">
         <f>J14</f>
         <v>6411-rt6</v>
       </c>
-      <c r="K21" s="9">
+      <c r="K21" s="11">
         <v>26.1</v>
       </c>
     </row>
     <row r="22" spans="7:11" x14ac:dyDescent="0.3">
-      <c r="G22" s="10" t="s">
+      <c r="G22" s="12" t="s">
         <v>13</v>
       </c>
-      <c r="H22" s="11" t="str">
+      <c r="H22" s="13" t="str">
         <f>"Classic_Reimagined_10" &amp; G19</f>
         <v>Classic_Reimagined_10_SE_2.1</v>
       </c>
-      <c r="I22" s="12"/>
-      <c r="J22" s="13"/>
-      <c r="K22" s="14"/>
+      <c r="I22" s="14"/>
+      <c r="J22" s="15"/>
+      <c r="K22" s="16"/>
     </row>
     <row r="23" spans="7:11" x14ac:dyDescent="0.3">
-      <c r="G23" s="10" t="s">
+      <c r="G23" s="12" t="s">
         <v>14</v>
       </c>
-      <c r="H23" s="11" t="str">
+      <c r="H23" s="13" t="str">
         <f>G21 &amp; "." &amp; H21 &amp; "_" &amp; I21 &amp; "-" &amp; H22</f>
         <v>v10.0.11_1-Classic_Reimagined_10_SE_2.1</v>
       </c>
-      <c r="I23" s="12"/>
-      <c r="J23" s="13"/>
-      <c r="K23" s="14"/>
+      <c r="I23" s="14"/>
+      <c r="J23" s="15"/>
+      <c r="K23" s="16"/>
     </row>
     <row r="24" spans="7:11" x14ac:dyDescent="0.3">
-      <c r="G24" s="10" t="s">
+      <c r="G24" s="12" t="s">
         <v>15</v>
       </c>
-      <c r="H24" s="11" t="str">
+      <c r="H24" s="13" t="str">
         <f>H23 &amp; "-build-" &amp; J21</f>
         <v>v10.0.11_1-Classic_Reimagined_10_SE_2.1-build-6411-rt6</v>
       </c>
-      <c r="I24" s="12"/>
-      <c r="J24" s="13"/>
+      <c r="I24" s="14"/>
+      <c r="J24" s="15"/>
     </row>
     <row r="25" spans="7:11" x14ac:dyDescent="0.3">
-      <c r="G25" s="7" t="s">
+      <c r="G25" s="9" t="s">
         <v>16</v>
       </c>
     </row>
     <row r="26" spans="7:11" x14ac:dyDescent="0.3">
-      <c r="G26" s="8" t="s">
+      <c r="G26" s="10" t="s">
         <v>17</v>
       </c>
-      <c r="H26" s="8" t="s">
+      <c r="H26" s="10" t="s">
         <v>6</v>
       </c>
-      <c r="I26" s="8" t="s">
+      <c r="I26" s="10" t="s">
         <v>3</v>
       </c>
-      <c r="J26" s="8" t="s">
+      <c r="J26" s="10" t="s">
         <v>4</v>
       </c>
     </row>
     <row r="27" spans="7:11" x14ac:dyDescent="0.3">
-      <c r="G27" s="9" t="s">
+      <c r="G27" s="11" t="s">
         <v>11</v>
       </c>
-      <c r="H27" s="9">
+      <c r="H27" s="11">
         <v>10</v>
       </c>
-      <c r="I27" s="9" t="str">
+      <c r="I27" s="11" t="str">
         <f>J21</f>
         <v>6411-rt6</v>
       </c>
-      <c r="J27" s="9" t="s">
+      <c r="J27" s="11" t="s">
         <v>18</v>
       </c>
     </row>
     <row r="28" spans="7:11" x14ac:dyDescent="0.3">
-      <c r="G28" s="10" t="s">
+      <c r="G28" s="12" t="s">
         <v>13</v>
       </c>
-      <c r="H28" s="15" t="str">
+      <c r="H28" s="22" t="str">
         <f>"Classic_Reimagined_10" &amp; G25</f>
         <v>Classic_Reimagined_10_SE_2</v>
       </c>
-      <c r="I28" s="16"/>
-      <c r="J28" s="14"/>
+      <c r="I28" s="23"/>
+      <c r="J28" s="16"/>
     </row>
     <row r="29" spans="7:11" x14ac:dyDescent="0.3">
-      <c r="G29" s="10" t="s">
+      <c r="G29" s="12" t="s">
         <v>14</v>
       </c>
-      <c r="H29" s="15" t="str">
+      <c r="H29" s="22" t="str">
         <f>G27 &amp; "." &amp; H27 &amp; "-" &amp; H28</f>
         <v>v10.0.10-Classic_Reimagined_10_SE_2</v>
       </c>
-      <c r="I29" s="16"/>
-      <c r="J29" s="14"/>
+      <c r="I29" s="23"/>
+      <c r="J29" s="16"/>
     </row>
     <row r="30" spans="7:11" x14ac:dyDescent="0.3">
-      <c r="G30" s="10" t="s">
+      <c r="G30" s="12" t="s">
         <v>15</v>
       </c>
-      <c r="H30" s="15" t="str">
+      <c r="H30" s="22" t="str">
         <f>H29 &amp; "-build-" &amp; I27</f>
         <v>v10.0.10-Classic_Reimagined_10_SE_2-build-6411-rt6</v>
       </c>
-      <c r="I30" s="16"/>
+      <c r="I30" s="23"/>
     </row>
     <row r="31" spans="7:11" x14ac:dyDescent="0.3">
-      <c r="G31" s="8" t="s">
+      <c r="G31" s="10" t="s">
         <v>17</v>
       </c>
-      <c r="H31" s="8" t="s">
+      <c r="H31" s="10" t="s">
         <v>6</v>
       </c>
-      <c r="I31" s="8" t="s">
+      <c r="I31" s="10" t="s">
         <v>3</v>
       </c>
-      <c r="J31" s="8" t="s">
+      <c r="J31" s="10" t="s">
         <v>4</v>
       </c>
     </row>
     <row r="32" spans="7:11" x14ac:dyDescent="0.3">
-      <c r="G32" s="9" t="s">
+      <c r="G32" s="11" t="s">
         <v>11</v>
       </c>
-      <c r="H32" s="9">
+      <c r="H32" s="11">
         <v>9</v>
       </c>
-      <c r="I32" s="9" t="str">
+      <c r="I32" s="11" t="str">
         <f>I27</f>
         <v>6411-rt6</v>
       </c>
-      <c r="J32" s="9" t="s">
+      <c r="J32" s="11" t="s">
         <v>19</v>
       </c>
     </row>
     <row r="33" spans="7:10" x14ac:dyDescent="0.3">
-      <c r="G33" s="10" t="s">
+      <c r="G33" s="12" t="s">
         <v>13</v>
       </c>
-      <c r="H33" s="15" t="str">
+      <c r="H33" s="22" t="str">
         <f>H28</f>
         <v>Classic_Reimagined_10_SE_2</v>
       </c>
-      <c r="I33" s="16"/>
-      <c r="J33" s="14"/>
+      <c r="I33" s="23"/>
+      <c r="J33" s="16"/>
     </row>
     <row r="34" spans="7:10" x14ac:dyDescent="0.3">
-      <c r="G34" s="10" t="s">
+      <c r="G34" s="12" t="s">
         <v>14</v>
       </c>
-      <c r="H34" s="15" t="str">
+      <c r="H34" s="22" t="str">
         <f>G32 &amp; "." &amp; H32 &amp; "-" &amp; H33</f>
         <v>v10.0.9-Classic_Reimagined_10_SE_2</v>
       </c>
-      <c r="I34" s="16"/>
-      <c r="J34" s="14"/>
+      <c r="I34" s="23"/>
+      <c r="J34" s="16"/>
     </row>
     <row r="35" spans="7:10" x14ac:dyDescent="0.3">
-      <c r="G35" s="10" t="s">
+      <c r="G35" s="12" t="s">
         <v>15</v>
       </c>
-      <c r="H35" s="15" t="str">
+      <c r="H35" s="22" t="str">
         <f>H34 &amp; "-build-" &amp; I32</f>
         <v>v10.0.9-Classic_Reimagined_10_SE_2-build-6411-rt6</v>
       </c>
-      <c r="I35" s="16"/>
+      <c r="I35" s="23"/>
     </row>
     <row r="36" spans="7:10" x14ac:dyDescent="0.3">
-      <c r="G36" s="8" t="s">
+      <c r="G36" s="10" t="s">
         <v>17</v>
       </c>
-      <c r="H36" s="8" t="s">
+      <c r="H36" s="10" t="s">
         <v>6</v>
       </c>
-      <c r="I36" s="8" t="s">
+      <c r="I36" s="10" t="s">
         <v>3</v>
       </c>
-      <c r="J36" s="8" t="s">
+      <c r="J36" s="10" t="s">
         <v>4</v>
       </c>
     </row>
     <row r="37" spans="7:10" x14ac:dyDescent="0.3">
-      <c r="G37" s="9" t="s">
+      <c r="G37" s="11" t="s">
         <v>11</v>
       </c>
-      <c r="H37" s="9">
+      <c r="H37" s="11">
         <v>7</v>
       </c>
-      <c r="I37" s="9" t="str">
+      <c r="I37" s="11" t="str">
         <f>I32</f>
         <v>6411-rt6</v>
       </c>
-      <c r="J37" s="9" t="s">
+      <c r="J37" s="11" t="s">
         <v>20</v>
       </c>
     </row>
     <row r="38" spans="7:10" x14ac:dyDescent="0.3">
-      <c r="G38" s="10" t="s">
+      <c r="G38" s="12" t="s">
         <v>13</v>
       </c>
-      <c r="H38" s="15" t="str">
+      <c r="H38" s="22" t="str">
         <f>H33</f>
         <v>Classic_Reimagined_10_SE_2</v>
       </c>
-      <c r="I38" s="16"/>
-      <c r="J38" s="14"/>
+      <c r="I38" s="23"/>
+      <c r="J38" s="16"/>
     </row>
     <row r="39" spans="7:10" x14ac:dyDescent="0.3">
-      <c r="G39" s="10" t="s">
+      <c r="G39" s="12" t="s">
         <v>14</v>
       </c>
-      <c r="H39" s="15" t="str">
+      <c r="H39" s="22" t="str">
         <f>G37 &amp; "." &amp; H37 &amp; "-" &amp; H38</f>
         <v>v10.0.7-Classic_Reimagined_10_SE_2</v>
       </c>
-      <c r="I39" s="16"/>
-      <c r="J39" s="14"/>
+      <c r="I39" s="23"/>
+      <c r="J39" s="16"/>
     </row>
     <row r="40" spans="7:10" x14ac:dyDescent="0.3">
-      <c r="G40" s="10" t="s">
+      <c r="G40" s="12" t="s">
         <v>15</v>
       </c>
-      <c r="H40" s="15" t="str">
+      <c r="H40" s="22" t="str">
         <f>H39 &amp; "-build-" &amp; I37</f>
         <v>v10.0.7-Classic_Reimagined_10_SE_2-build-6411-rt6</v>
       </c>
-      <c r="I40" s="16"/>
+      <c r="I40" s="23"/>
     </row>
     <row r="41" spans="7:10" x14ac:dyDescent="0.3">
-      <c r="G41" s="8" t="s">
+      <c r="G41" s="10" t="s">
         <v>17</v>
       </c>
-      <c r="H41" s="8" t="s">
+      <c r="H41" s="10" t="s">
         <v>6</v>
       </c>
-      <c r="I41" s="8" t="s">
+      <c r="I41" s="10" t="s">
         <v>3</v>
       </c>
-      <c r="J41" s="8" t="s">
+      <c r="J41" s="10" t="s">
         <v>4</v>
       </c>
     </row>
     <row r="42" spans="7:10" x14ac:dyDescent="0.3">
-      <c r="G42" s="9" t="s">
+      <c r="G42" s="11" t="s">
         <v>11</v>
       </c>
-      <c r="H42" s="9">
-        <v>4</v>
-      </c>
-      <c r="I42" s="9" t="str">
+      <c r="H42" s="11">
+        <v>4</v>
+      </c>
+      <c r="I42" s="11" t="str">
         <f>I37</f>
         <v>6411-rt6</v>
       </c>
-      <c r="J42" s="9" t="s">
+      <c r="J42" s="11" t="s">
         <v>21</v>
       </c>
     </row>
     <row r="43" spans="7:10" x14ac:dyDescent="0.3">
-      <c r="G43" s="10" t="s">
+      <c r="G43" s="12" t="s">
         <v>13</v>
       </c>
-      <c r="H43" s="15" t="str">
+      <c r="H43" s="22" t="str">
         <f>H38</f>
         <v>Classic_Reimagined_10_SE_2</v>
       </c>
-      <c r="I43" s="16"/>
-      <c r="J43" s="14"/>
+      <c r="I43" s="23"/>
+      <c r="J43" s="16"/>
     </row>
     <row r="44" spans="7:10" x14ac:dyDescent="0.3">
-      <c r="G44" s="10" t="s">
+      <c r="G44" s="12" t="s">
         <v>14</v>
       </c>
-      <c r="H44" s="15" t="str">
+      <c r="H44" s="22" t="str">
         <f>G42 &amp; "." &amp; H42 &amp; "-" &amp; H43</f>
         <v>v10.0.4-Classic_Reimagined_10_SE_2</v>
       </c>
-      <c r="I44" s="16"/>
-      <c r="J44" s="14"/>
+      <c r="I44" s="23"/>
+      <c r="J44" s="16"/>
     </row>
     <row r="45" spans="7:10" x14ac:dyDescent="0.3">
-      <c r="G45" s="10" t="s">
+      <c r="G45" s="12" t="s">
         <v>15</v>
       </c>
-      <c r="H45" s="15" t="str">
+      <c r="H45" s="22" t="str">
         <f>H44 &amp; "-build-" &amp; I42</f>
         <v>v10.0.4-Classic_Reimagined_10_SE_2-build-6411-rt6</v>
       </c>
-      <c r="I45" s="16"/>
+      <c r="I45" s="23"/>
     </row>
     <row r="46" spans="7:10" x14ac:dyDescent="0.3">
-      <c r="G46" s="7" t="s">
+      <c r="G46" s="9" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="47" spans="7:10" x14ac:dyDescent="0.3">
-      <c r="G47" s="8" t="s">
+      <c r="G47" s="10" t="s">
         <v>17</v>
       </c>
-      <c r="H47" s="8" t="s">
+      <c r="H47" s="10" t="s">
         <v>6</v>
       </c>
-      <c r="I47" s="8" t="s">
+      <c r="I47" s="10" t="s">
         <v>3</v>
       </c>
-      <c r="J47" s="8" t="s">
+      <c r="J47" s="10" t="s">
         <v>4</v>
       </c>
     </row>
     <row r="48" spans="7:10" x14ac:dyDescent="0.3">
-      <c r="G48" s="9" t="s">
+      <c r="G48" s="11" t="s">
         <v>11</v>
       </c>
-      <c r="H48" s="9">
+      <c r="H48" s="11">
         <v>3</v>
       </c>
-      <c r="I48" s="9" t="str">
+      <c r="I48" s="11" t="str">
         <f>I42</f>
         <v>6411-rt6</v>
       </c>
-      <c r="J48" s="9" t="s">
+      <c r="J48" s="11" t="s">
         <v>23</v>
       </c>
     </row>
     <row r="49" spans="7:10" x14ac:dyDescent="0.3">
-      <c r="G49" s="10" t="s">
+      <c r="G49" s="12" t="s">
         <v>13</v>
       </c>
-      <c r="H49" s="15" t="str">
+      <c r="H49" s="22" t="str">
         <f>"Classic_Reimagined_10" &amp; G46</f>
         <v>Classic_Reimagined_10_SE</v>
       </c>
-      <c r="I49" s="16"/>
-      <c r="J49" s="14"/>
+      <c r="I49" s="23"/>
+      <c r="J49" s="16"/>
     </row>
     <row r="50" spans="7:10" x14ac:dyDescent="0.3">
-      <c r="G50" s="10" t="s">
+      <c r="G50" s="12" t="s">
         <v>14</v>
       </c>
-      <c r="H50" s="15" t="str">
+      <c r="H50" s="22" t="str">
         <f>G48 &amp; "." &amp; H48 &amp; "-" &amp; H49</f>
         <v>v10.0.3-Classic_Reimagined_10_SE</v>
       </c>
-      <c r="I50" s="16"/>
-      <c r="J50" s="14"/>
+      <c r="I50" s="23"/>
+      <c r="J50" s="16"/>
     </row>
     <row r="51" spans="7:10" x14ac:dyDescent="0.3">
-      <c r="G51" s="10" t="s">
+      <c r="G51" s="12" t="s">
         <v>15</v>
       </c>
-      <c r="H51" s="15" t="str">
+      <c r="H51" s="22" t="str">
         <f>H50 &amp; "-build-" &amp; I48</f>
         <v>v10.0.3-Classic_Reimagined_10_SE-build-6411-rt6</v>
       </c>
-      <c r="I51" s="16"/>
+      <c r="I51" s="23"/>
     </row>
     <row r="52" spans="7:10" x14ac:dyDescent="0.3">
-      <c r="G52" s="7" t="s">
+      <c r="G52" s="9" t="s">
         <v>24</v>
       </c>
     </row>
     <row r="53" spans="7:10" x14ac:dyDescent="0.3">
-      <c r="G53" s="8" t="s">
+      <c r="G53" s="10" t="s">
         <v>17</v>
       </c>
-      <c r="H53" s="8" t="s">
+      <c r="H53" s="10" t="s">
         <v>6</v>
       </c>
-      <c r="I53" s="8" t="s">
+      <c r="I53" s="10" t="s">
         <v>3</v>
       </c>
-      <c r="J53" s="8" t="s">
+      <c r="J53" s="10" t="s">
         <v>4</v>
       </c>
     </row>
     <row r="54" spans="7:10" x14ac:dyDescent="0.3">
-      <c r="G54" s="9" t="s">
+      <c r="G54" s="11" t="s">
         <v>11</v>
       </c>
-      <c r="H54" s="9">
+      <c r="H54" s="11">
         <v>2</v>
       </c>
-      <c r="I54" s="9" t="str">
+      <c r="I54" s="11" t="str">
         <f>I48</f>
         <v>6411-rt6</v>
       </c>
-      <c r="J54" s="9" t="s">
+      <c r="J54" s="11" t="s">
         <v>25</v>
       </c>
     </row>
     <row r="55" spans="7:10" x14ac:dyDescent="0.3">
-      <c r="G55" s="10" t="s">
+      <c r="G55" s="12" t="s">
         <v>13</v>
       </c>
-      <c r="H55" s="15" t="s">
+      <c r="H55" s="22" t="s">
         <v>26</v>
       </c>
-      <c r="I55" s="16"/>
-      <c r="J55" s="14"/>
+      <c r="I55" s="23"/>
+      <c r="J55" s="16"/>
     </row>
     <row r="56" spans="7:10" x14ac:dyDescent="0.3">
-      <c r="G56" s="10" t="s">
+      <c r="G56" s="12" t="s">
         <v>14</v>
       </c>
-      <c r="H56" s="15" t="str">
+      <c r="H56" s="22" t="str">
         <f>G54 &amp; "." &amp; H54 &amp; "-" &amp; H55</f>
         <v>v10.0.2-Classic_Reimagined_10s</v>
       </c>
-      <c r="I56" s="16"/>
-      <c r="J56" s="14"/>
+      <c r="I56" s="23"/>
+      <c r="J56" s="16"/>
     </row>
     <row r="57" spans="7:10" x14ac:dyDescent="0.3">
-      <c r="G57" s="10" t="s">
+      <c r="G57" s="12" t="s">
         <v>15</v>
       </c>
-      <c r="H57" s="15" t="str">
+      <c r="H57" s="22" t="str">
         <f>H56 &amp; "-build-" &amp; I54</f>
         <v>v10.0.2-Classic_Reimagined_10s-build-6411-rt6</v>
       </c>
-      <c r="I57" s="16"/>
+      <c r="I57" s="23"/>
     </row>
     <row r="58" spans="7:10" x14ac:dyDescent="0.3">
-      <c r="G58" s="7" t="s">
+      <c r="G58" s="9" t="s">
         <v>27</v>
       </c>
     </row>
     <row r="59" spans="7:10" x14ac:dyDescent="0.3">
-      <c r="G59" s="8" t="s">
+      <c r="G59" s="10" t="s">
         <v>17</v>
       </c>
-      <c r="H59" s="8" t="s">
+      <c r="H59" s="10" t="s">
         <v>6</v>
       </c>
-      <c r="I59" s="8" t="s">
+      <c r="I59" s="10" t="s">
         <v>3</v>
       </c>
-      <c r="J59" s="8" t="s">
+      <c r="J59" s="10" t="s">
         <v>4</v>
       </c>
     </row>
     <row r="60" spans="7:10" x14ac:dyDescent="0.3">
-      <c r="G60" s="9" t="s">
+      <c r="G60" s="11" t="s">
         <v>11</v>
       </c>
-      <c r="H60" s="9">
+      <c r="H60" s="11">
         <v>1</v>
       </c>
-      <c r="I60" s="9" t="str">
+      <c r="I60" s="11" t="str">
         <f>I54</f>
         <v>6411-rt6</v>
       </c>
-      <c r="J60" s="9" t="s">
+      <c r="J60" s="11" t="s">
         <v>28</v>
       </c>
     </row>
     <row r="61" spans="7:10" x14ac:dyDescent="0.3">
-      <c r="G61" s="10" t="s">
+      <c r="G61" s="12" t="s">
         <v>13</v>
       </c>
-      <c r="H61" s="15" t="s">
+      <c r="H61" s="22" t="s">
         <v>29</v>
       </c>
-      <c r="I61" s="16"/>
-      <c r="J61" s="14"/>
+      <c r="I61" s="23"/>
+      <c r="J61" s="16"/>
     </row>
     <row r="62" spans="7:10" x14ac:dyDescent="0.3">
-      <c r="G62" s="10" t="s">
+      <c r="G62" s="12" t="s">
         <v>14</v>
       </c>
-      <c r="H62" s="15" t="str">
+      <c r="H62" s="22" t="str">
         <f>G60 &amp; "." &amp; H60 &amp; "-" &amp; H61</f>
         <v>v10.0.1-Classic_Reimagined_10</v>
       </c>
-      <c r="I62" s="16"/>
-      <c r="J62" s="14"/>
+      <c r="I62" s="23"/>
+      <c r="J62" s="16"/>
     </row>
     <row r="63" spans="7:10" x14ac:dyDescent="0.3">
-      <c r="G63" s="10" t="s">
+      <c r="G63" s="12" t="s">
         <v>15</v>
       </c>
-      <c r="H63" s="15" t="str">
+      <c r="H63" s="22" t="str">
         <f>H62 &amp; "-build-" &amp; I60</f>
         <v>v10.0.1-Classic_Reimagined_10-build-6411-rt6</v>
       </c>
-      <c r="I63" s="16"/>
+      <c r="I63" s="23"/>
     </row>
     <row r="64" spans="7:10" x14ac:dyDescent="0.3">
       <c r="G64" s="24" t="s">
@@ -1595,134 +1600,134 @@
       <c r="J64" s="24"/>
     </row>
     <row r="65" spans="7:10" x14ac:dyDescent="0.3">
-      <c r="G65" s="7" t="s">
+      <c r="G65" s="9" t="s">
         <v>31</v>
       </c>
     </row>
     <row r="66" spans="7:10" x14ac:dyDescent="0.3">
-      <c r="G66" s="8" t="s">
+      <c r="G66" s="10" t="s">
         <v>17</v>
       </c>
-      <c r="H66" s="8" t="s">
+      <c r="H66" s="10" t="s">
         <v>6</v>
       </c>
-      <c r="I66" s="8" t="s">
+      <c r="I66" s="10" t="s">
         <v>3</v>
       </c>
-      <c r="J66" s="8" t="s">
+      <c r="J66" s="10" t="s">
         <v>4</v>
       </c>
     </row>
     <row r="67" spans="7:10" x14ac:dyDescent="0.3">
-      <c r="G67" s="9" t="s">
+      <c r="G67" s="11" t="s">
         <v>32</v>
       </c>
-      <c r="H67" s="9">
+      <c r="H67" s="11">
         <v>32</v>
       </c>
-      <c r="I67" s="9" t="str">
+      <c r="I67" s="11" t="str">
         <f>I60</f>
         <v>6411-rt6</v>
       </c>
-      <c r="J67" s="9" t="s">
+      <c r="J67" s="11" t="s">
         <v>33</v>
       </c>
     </row>
     <row r="68" spans="7:10" x14ac:dyDescent="0.3">
-      <c r="G68" s="10" t="s">
+      <c r="G68" s="12" t="s">
         <v>13</v>
       </c>
-      <c r="H68" s="15" t="s">
+      <c r="H68" s="22" t="s">
         <v>34</v>
       </c>
-      <c r="I68" s="16"/>
-      <c r="J68" s="14"/>
+      <c r="I68" s="23"/>
+      <c r="J68" s="16"/>
     </row>
     <row r="69" spans="7:10" x14ac:dyDescent="0.3">
-      <c r="G69" s="10" t="s">
+      <c r="G69" s="12" t="s">
         <v>14</v>
       </c>
-      <c r="H69" s="15" t="str">
+      <c r="H69" s="22" t="str">
         <f>G67 &amp; "." &amp; H67 &amp; "-" &amp; H68</f>
         <v>v8.10.32-Classic_Reimagined_8</v>
       </c>
-      <c r="I69" s="16"/>
-      <c r="J69" s="14"/>
+      <c r="I69" s="23"/>
+      <c r="J69" s="16"/>
     </row>
     <row r="70" spans="7:10" x14ac:dyDescent="0.3">
-      <c r="G70" s="10" t="s">
+      <c r="G70" s="12" t="s">
         <v>15</v>
       </c>
-      <c r="H70" s="15" t="str">
+      <c r="H70" s="22" t="str">
         <f>H69 &amp; "-build-" &amp; I67</f>
         <v>v8.10.32-Classic_Reimagined_8-build-6411-rt6</v>
       </c>
-      <c r="I70" s="16"/>
+      <c r="I70" s="23"/>
     </row>
     <row r="71" spans="7:10" x14ac:dyDescent="0.3">
-      <c r="G71" s="7" t="s">
+      <c r="G71" s="9" t="s">
         <v>31</v>
       </c>
     </row>
     <row r="72" spans="7:10" x14ac:dyDescent="0.3">
-      <c r="G72" s="8" t="s">
+      <c r="G72" s="10" t="s">
         <v>17</v>
       </c>
-      <c r="H72" s="8" t="s">
+      <c r="H72" s="10" t="s">
         <v>6</v>
       </c>
-      <c r="I72" s="8" t="s">
+      <c r="I72" s="10" t="s">
         <v>3</v>
       </c>
-      <c r="J72" s="8" t="s">
+      <c r="J72" s="10" t="s">
         <v>4</v>
       </c>
     </row>
     <row r="73" spans="7:10" x14ac:dyDescent="0.3">
-      <c r="G73" s="9" t="s">
+      <c r="G73" s="11" t="s">
         <v>32</v>
       </c>
-      <c r="H73" s="9">
+      <c r="H73" s="11">
         <v>31</v>
       </c>
-      <c r="I73" s="9" t="str">
+      <c r="I73" s="11" t="str">
         <f>I67</f>
         <v>6411-rt6</v>
       </c>
-      <c r="J73" s="9" t="s">
+      <c r="J73" s="11" t="s">
         <v>35</v>
       </c>
     </row>
     <row r="74" spans="7:10" x14ac:dyDescent="0.3">
-      <c r="G74" s="10" t="s">
+      <c r="G74" s="12" t="s">
         <v>13</v>
       </c>
-      <c r="H74" s="15" t="s">
+      <c r="H74" s="22" t="s">
         <v>34</v>
       </c>
-      <c r="I74" s="16"/>
-      <c r="J74" s="14"/>
+      <c r="I74" s="23"/>
+      <c r="J74" s="16"/>
     </row>
     <row r="75" spans="7:10" x14ac:dyDescent="0.3">
-      <c r="G75" s="10" t="s">
+      <c r="G75" s="12" t="s">
         <v>14</v>
       </c>
-      <c r="H75" s="15" t="str">
+      <c r="H75" s="22" t="str">
         <f>G73 &amp; "." &amp; H73 &amp; "-" &amp; H74</f>
         <v>v8.10.31-Classic_Reimagined_8</v>
       </c>
-      <c r="I75" s="16"/>
-      <c r="J75" s="14"/>
+      <c r="I75" s="23"/>
+      <c r="J75" s="16"/>
     </row>
     <row r="76" spans="7:10" x14ac:dyDescent="0.3">
-      <c r="G76" s="10" t="s">
+      <c r="G76" s="12" t="s">
         <v>15</v>
       </c>
-      <c r="H76" s="15" t="str">
+      <c r="H76" s="22" t="str">
         <f>H75 &amp; "-build-" &amp; I73</f>
         <v>v8.10.31-Classic_Reimagined_8-build-6411-rt6</v>
       </c>
-      <c r="I76" s="16"/>
+      <c r="I76" s="23"/>
     </row>
     <row r="77" spans="7:10" x14ac:dyDescent="0.3">
       <c r="G77" s="25" t="s">
@@ -1733,64 +1738,64 @@
       <c r="J77" s="25"/>
     </row>
     <row r="78" spans="7:10" x14ac:dyDescent="0.3">
-      <c r="G78" s="8" t="s">
+      <c r="G78" s="10" t="s">
         <v>17</v>
       </c>
-      <c r="H78" s="8" t="s">
+      <c r="H78" s="10" t="s">
         <v>6</v>
       </c>
-      <c r="I78" s="8" t="s">
+      <c r="I78" s="10" t="s">
         <v>3</v>
       </c>
-      <c r="J78" s="8" t="s">
+      <c r="J78" s="10" t="s">
         <v>4</v>
       </c>
     </row>
     <row r="79" spans="7:10" x14ac:dyDescent="0.3">
-      <c r="G79" s="9" t="s">
+      <c r="G79" s="11" t="s">
         <v>37</v>
       </c>
-      <c r="H79" s="9">
+      <c r="H79" s="11">
         <v>3</v>
       </c>
-      <c r="I79" s="9" t="str">
+      <c r="I79" s="11" t="str">
         <f>I73</f>
         <v>6411-rt6</v>
       </c>
-      <c r="J79" s="9" t="s">
+      <c r="J79" s="11" t="s">
         <v>38</v>
       </c>
     </row>
     <row r="80" spans="7:10" x14ac:dyDescent="0.3">
-      <c r="G80" s="10" t="s">
+      <c r="G80" s="12" t="s">
         <v>13</v>
       </c>
-      <c r="H80" s="15" t="s">
+      <c r="H80" s="22" t="s">
         <v>39</v>
       </c>
-      <c r="I80" s="16"/>
-      <c r="J80" s="14"/>
+      <c r="I80" s="23"/>
+      <c r="J80" s="16"/>
     </row>
     <row r="81" spans="7:10" x14ac:dyDescent="0.3">
-      <c r="G81" s="10" t="s">
+      <c r="G81" s="12" t="s">
         <v>14</v>
       </c>
-      <c r="H81" s="15" t="str">
+      <c r="H81" s="22" t="str">
         <f>G79 &amp; "." &amp; H79 &amp; "-" &amp; H80</f>
         <v>v7.11.3-Better_Default_7</v>
       </c>
-      <c r="I81" s="16"/>
-      <c r="J81" s="14"/>
+      <c r="I81" s="23"/>
+      <c r="J81" s="16"/>
     </row>
     <row r="82" spans="7:10" x14ac:dyDescent="0.3">
-      <c r="G82" s="10" t="s">
+      <c r="G82" s="12" t="s">
         <v>15</v>
       </c>
-      <c r="H82" s="15" t="str">
+      <c r="H82" s="22" t="str">
         <f>H81 &amp; "-build-" &amp; I79</f>
         <v>v7.11.3-Better_Default_7-build-6411-rt6</v>
       </c>
-      <c r="I82" s="16"/>
+      <c r="I82" s="23"/>
     </row>
   </sheetData>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A10:A24">

</xml_diff>